<commit_message>
Fix legally problematic clauses across documents
- 重要事項説明書: drop expired 処遇改善加算(Ⅴ), fix inverted cancellation fees
- 契約書: align payment date and arrears notice with 重要事項説明書
- 休暇規程/育児・介護休業規程: annual leave per tenure, 2025 amendments, hourly leave, statutory leaves
- 安全衛生規程: 衛生推進者 appointment is mandatory
- 懲戒規程: 禁錮 -> 拘禁刑
- 福利厚生規程: meal allowance not limited to full-time staff
- 退職規程: retirement age, dismissal notice, wage settlement, installment consent

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019FEKn7HFzGRhKMsA45fWaY
</commit_message>
<xml_diff>
--- a/output/いいかいご_契約書類一式.xlsx
+++ b/output/いいかいご_契約書類一式.xlsx
@@ -2028,7 +2028,7 @@
         </is>
       </c>
     </row>
-    <row r="103" ht="750" customHeight="1">
+    <row r="103" ht="120" customHeight="1">
       <c r="A103" s="6" t="inlineStr">
         <is>
           <t>介護職員等処遇改善加算
@@ -2041,21 +2041,7 @@
           <t>（Ⅰ）所定単位数の245/1000
 （Ⅱ）所定単位数の224/1000
 （Ⅲ）所定単位数の182/1000
-（Ⅳ）所定単位数の145/1000
-（Ⅴ1）所定単位数の221/1000
-（Ⅴ2）所定単位数の208/1000
-（Ⅴ3）所定単位数の200/1000
-（Ⅴ4）所定単位数の187/1000
-（Ⅴ5）所定単位数の184/1000
-（Ⅴ6）所定単位数の163/1000
-（Ⅴ7）所定単位数の163/1000
-（Ⅴ8）所定単位数の158/1000
-（Ⅴ9）所定単位数の142/1000
-（Ⅴ10）所定単位数の139/1000
-（Ⅴ11）所定単位数の121/1000
-（Ⅴ12）所定単位数の118/1000
-（Ⅴ13）所定単位数の100/1000
-（Ⅴ14）所定単位数の76/1000</t>
+（Ⅳ）所定単位数の145/1000</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
@@ -2065,8 +2051,7 @@
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>基本サービス費に各種加算減算を加えた総単位数（所定単位数）
-※（Ⅴ）は令和7年3月31日まで算定可</t>
+          <t>基本サービス費に各種加算減算を加えた総単位数（所定単位数）</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2320,7 @@
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>１提供当たりの料金の100%を請求いたします。</t>
+          <t>１提供当たりの利用者負担額の50%を請求いたします。</t>
         </is>
       </c>
       <c r="D141" s="4" t="n"/>
@@ -2354,7 +2339,7 @@
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>１提供当たりの料金の50%を請求いたします。</t>
+          <t>１提供当たりの利用者負担額の100%を請求いたします。</t>
         </is>
       </c>
       <c r="D142" s="4" t="n"/>
@@ -3593,7 +3578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E192"/>
+  <dimension ref="A1:E193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -4293,331 +4278,341 @@
     <row r="132" ht="20" customHeight="1">
       <c r="A132" s="27" t="inlineStr">
         <is>
-          <t>第16条　会社は、正社員に対し、一律月額10,000円の食事補助手当を支給する。</t>
-        </is>
-      </c>
-    </row>
-    <row r="133" ht="8" customHeight="1"/>
-    <row r="134" ht="20" customHeight="1">
-      <c r="A134" s="26" t="inlineStr">
+          <t>第16条　会社は、従業員に対し、月額10,000円の食事補助手当を支給する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="32" customHeight="1">
+      <c r="A133" s="27" t="inlineStr">
+        <is>
+          <t>2　パートタイマー等の所定労働日数が少ない従業員については、出勤日数に応じて按分して支給する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="8" customHeight="1"/>
+    <row r="135" ht="20" customHeight="1">
+      <c r="A135" s="26" t="inlineStr">
         <is>
           <t>（制服・作業着）</t>
-        </is>
-      </c>
-    </row>
-    <row r="135" ht="32" customHeight="1">
-      <c r="A135" s="27" t="inlineStr">
-        <is>
-          <t>第17条　従業員は、業務に従事するにあたり会社が指定する制服または作業着を着用しなければならない。</t>
         </is>
       </c>
     </row>
     <row r="136" ht="32" customHeight="1">
       <c r="A136" s="27" t="inlineStr">
         <is>
+          <t>第17条　従業員は、業務に従事するにあたり会社が指定する制服または作業着を着用しなければならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="32" customHeight="1">
+      <c r="A137" s="27" t="inlineStr">
+        <is>
           <t>2　制服または作業着は、原則として従業員が自ら準備するものとする。ただし、会社が特に必要と認めた場合は、会社が貸与または支給することがある。</t>
         </is>
       </c>
     </row>
-    <row r="137" ht="8" customHeight="1"/>
-    <row r="138" ht="20" customHeight="1">
-      <c r="A138" s="26" t="inlineStr">
+    <row r="138" ht="8" customHeight="1"/>
+    <row r="139" ht="20" customHeight="1">
+      <c r="A139" s="26" t="inlineStr">
         <is>
           <t>（慶弔給付）</t>
-        </is>
-      </c>
-    </row>
-    <row r="139" ht="20" customHeight="1">
-      <c r="A139" s="27" t="inlineStr">
-        <is>
-          <t>第18条　会社は、休暇規程に定める慶弔休暇に関連して、次の給付を行う。</t>
         </is>
       </c>
     </row>
     <row r="140" ht="20" customHeight="1">
       <c r="A140" s="27" t="inlineStr">
         <is>
-          <t>1　結婚祝い金：30,000円</t>
+          <t>第18条　会社は、休暇規程に定める慶弔休暇に関連して、次の給付を行う。</t>
         </is>
       </c>
     </row>
     <row r="141" ht="20" customHeight="1">
       <c r="A141" s="27" t="inlineStr">
         <is>
-          <t>2　出産祝い金：30,000円</t>
+          <t>1　結婚祝い金：30,000円</t>
         </is>
       </c>
     </row>
     <row r="142" ht="20" customHeight="1">
       <c r="A142" s="27" t="inlineStr">
         <is>
-          <t>3　弔事：本人または家族の希望に応じ、生花を手配する。</t>
+          <t>2　出産祝い金：30,000円</t>
         </is>
       </c>
     </row>
     <row r="143" ht="20" customHeight="1">
       <c r="A143" s="27" t="inlineStr">
         <is>
+          <t>3　弔事：本人または家族の希望に応じ、生花を手配する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="20" customHeight="1">
+      <c r="A144" s="27" t="inlineStr">
+        <is>
           <t>4　災害見舞金：取締役会の判断により、最大100,000円を限度として支給する。</t>
         </is>
       </c>
     </row>
-    <row r="144" ht="8" customHeight="1"/>
-    <row r="145" ht="8" customHeight="1">
-      <c r="A145" s="28" t="inlineStr"/>
-      <c r="B145" s="12" t="n"/>
-      <c r="C145" s="12" t="n"/>
-      <c r="D145" s="12" t="n"/>
-      <c r="E145" s="12" t="n"/>
-    </row>
-    <row r="146" ht="10" customHeight="1"/>
-    <row r="147" ht="30" customHeight="1">
-      <c r="A147" s="25" t="inlineStr">
+    <row r="145" ht="8" customHeight="1"/>
+    <row r="146" ht="8" customHeight="1">
+      <c r="A146" s="28" t="inlineStr"/>
+      <c r="B146" s="12" t="n"/>
+      <c r="C146" s="12" t="n"/>
+      <c r="D146" s="12" t="n"/>
+      <c r="E146" s="12" t="n"/>
+    </row>
+    <row r="147" ht="10" customHeight="1"/>
+    <row r="148" ht="30" customHeight="1">
+      <c r="A148" s="25" t="inlineStr">
         <is>
           <t>第7章　健康・医療支援</t>
         </is>
       </c>
     </row>
-    <row r="148" ht="20" customHeight="1">
-      <c r="A148" s="26" t="inlineStr">
+    <row r="149" ht="20" customHeight="1">
+      <c r="A149" s="26" t="inlineStr">
         <is>
           <t>（健康診断）</t>
         </is>
       </c>
     </row>
-    <row r="149" ht="32" customHeight="1">
-      <c r="A149" s="27" t="inlineStr">
+    <row r="150" ht="32" customHeight="1">
+      <c r="A150" s="27" t="inlineStr">
         <is>
           <t>第19条　会社は、労働安全衛生法に基づき、従業員に対し年1回の健康診断を実施し、費用を会社が負担する。</t>
         </is>
       </c>
     </row>
-    <row r="150" ht="20" customHeight="1">
-      <c r="A150" s="27" t="inlineStr">
+    <row r="151" ht="20" customHeight="1">
+      <c r="A151" s="27" t="inlineStr">
         <is>
           <t>2　夜勤に従事する従業員については、年2回実施し、費用は会社が負担する。</t>
         </is>
       </c>
     </row>
-    <row r="151" ht="8" customHeight="1"/>
-    <row r="152" ht="8" customHeight="1">
-      <c r="A152" s="28" t="inlineStr"/>
-      <c r="B152" s="12" t="n"/>
-      <c r="C152" s="12" t="n"/>
-      <c r="D152" s="12" t="n"/>
-      <c r="E152" s="12" t="n"/>
-    </row>
-    <row r="153" ht="10" customHeight="1"/>
-    <row r="154" ht="30" customHeight="1">
-      <c r="A154" s="25" t="inlineStr">
+    <row r="152" ht="8" customHeight="1"/>
+    <row r="153" ht="8" customHeight="1">
+      <c r="A153" s="28" t="inlineStr"/>
+      <c r="B153" s="12" t="n"/>
+      <c r="C153" s="12" t="n"/>
+      <c r="D153" s="12" t="n"/>
+      <c r="E153" s="12" t="n"/>
+    </row>
+    <row r="154" ht="10" customHeight="1"/>
+    <row r="155" ht="30" customHeight="1">
+      <c r="A155" s="25" t="inlineStr">
         <is>
           <t>第8章　教育研修</t>
         </is>
       </c>
     </row>
-    <row r="155" ht="20" customHeight="1">
-      <c r="A155" s="26" t="inlineStr">
+    <row r="156" ht="20" customHeight="1">
+      <c r="A156" s="26" t="inlineStr">
         <is>
           <t>（外部研修）</t>
         </is>
       </c>
     </row>
-    <row r="156" ht="20" customHeight="1">
-      <c r="A156" s="27" t="inlineStr">
+    <row r="157" ht="20" customHeight="1">
+      <c r="A157" s="27" t="inlineStr">
         <is>
           <t>第20条　会社は、業務に資すると判断される外部研修について、参加費用を全額負担する。</t>
         </is>
       </c>
     </row>
-    <row r="157" ht="8" customHeight="1"/>
-    <row r="158" ht="8" customHeight="1">
-      <c r="A158" s="28" t="inlineStr"/>
-      <c r="B158" s="12" t="n"/>
-      <c r="C158" s="12" t="n"/>
-      <c r="D158" s="12" t="n"/>
-      <c r="E158" s="12" t="n"/>
-    </row>
-    <row r="159" ht="10" customHeight="1"/>
-    <row r="160" ht="30" customHeight="1">
-      <c r="A160" s="25" t="inlineStr">
+    <row r="158" ht="8" customHeight="1"/>
+    <row r="159" ht="8" customHeight="1">
+      <c r="A159" s="28" t="inlineStr"/>
+      <c r="B159" s="12" t="n"/>
+      <c r="C159" s="12" t="n"/>
+      <c r="D159" s="12" t="n"/>
+      <c r="E159" s="12" t="n"/>
+    </row>
+    <row r="160" ht="10" customHeight="1"/>
+    <row r="161" ht="30" customHeight="1">
+      <c r="A161" s="25" t="inlineStr">
         <is>
           <t>第9章　特別休暇に関連する給付</t>
         </is>
       </c>
     </row>
-    <row r="161" ht="20" customHeight="1">
-      <c r="A161" s="26" t="inlineStr">
+    <row r="162" ht="20" customHeight="1">
+      <c r="A162" s="26" t="inlineStr">
         <is>
           <t>（誕生日休暇・手当）</t>
         </is>
       </c>
     </row>
-    <row r="162" ht="32" customHeight="1">
-      <c r="A162" s="27" t="inlineStr">
+    <row r="163" ht="32" customHeight="1">
+      <c r="A163" s="27" t="inlineStr">
         <is>
           <t>第21条　会社は、休暇規程に基づき誕生日休暇を付与するとともに、当該休暇を取得した従業員に対して誕生日手当として10,000円を支給する。</t>
         </is>
       </c>
     </row>
-    <row r="163" ht="8" customHeight="1"/>
-    <row r="164" ht="20" customHeight="1">
-      <c r="A164" s="26" t="inlineStr">
+    <row r="164" ht="8" customHeight="1"/>
+    <row r="165" ht="20" customHeight="1">
+      <c r="A165" s="26" t="inlineStr">
         <is>
           <t>（特別休暇に伴う給付）</t>
         </is>
       </c>
     </row>
-    <row r="165" ht="32" customHeight="1">
-      <c r="A165" s="27" t="inlineStr">
+    <row r="166" ht="32" customHeight="1">
+      <c r="A166" s="27" t="inlineStr">
         <is>
           <t>第22条　会社は、休暇規程に基づき付与される特別休暇について、必要に応じて記念品、金銭その他の給付を行うことができる。内容は取締役会の決議により定める。</t>
         </is>
       </c>
     </row>
-    <row r="166" ht="8" customHeight="1"/>
-    <row r="167" ht="8" customHeight="1">
-      <c r="A167" s="28" t="inlineStr"/>
-      <c r="B167" s="12" t="n"/>
-      <c r="C167" s="12" t="n"/>
-      <c r="D167" s="12" t="n"/>
-      <c r="E167" s="12" t="n"/>
-    </row>
-    <row r="168" ht="10" customHeight="1"/>
-    <row r="169" ht="30" customHeight="1">
-      <c r="A169" s="25" t="inlineStr">
+    <row r="167" ht="8" customHeight="1"/>
+    <row r="168" ht="8" customHeight="1">
+      <c r="A168" s="28" t="inlineStr"/>
+      <c r="B168" s="12" t="n"/>
+      <c r="C168" s="12" t="n"/>
+      <c r="D168" s="12" t="n"/>
+      <c r="E168" s="12" t="n"/>
+    </row>
+    <row r="169" ht="10" customHeight="1"/>
+    <row r="170" ht="30" customHeight="1">
+      <c r="A170" s="25" t="inlineStr">
         <is>
           <t>第10章　運用</t>
         </is>
       </c>
     </row>
-    <row r="170" ht="20" customHeight="1">
-      <c r="A170" s="26" t="inlineStr">
+    <row r="171" ht="20" customHeight="1">
+      <c r="A171" s="26" t="inlineStr">
         <is>
           <t>（支給方法）</t>
         </is>
       </c>
     </row>
-    <row r="171" ht="32" customHeight="1">
-      <c r="A171" s="27" t="inlineStr">
+    <row r="172" ht="32" customHeight="1">
+      <c r="A172" s="27" t="inlineStr">
         <is>
           <t>第23条　通勤手当、特別通勤手当及び各種手当は、毎月1日から末日までの1か月分を集計し、当月の給与と併せて支給する。</t>
         </is>
       </c>
     </row>
-    <row r="172" ht="8" customHeight="1"/>
-    <row r="173" ht="20" customHeight="1">
-      <c r="A173" s="26" t="inlineStr">
+    <row r="173" ht="8" customHeight="1"/>
+    <row r="174" ht="20" customHeight="1">
+      <c r="A174" s="26" t="inlineStr">
         <is>
           <t>（中途入社・退職時の取扱い）</t>
         </is>
       </c>
     </row>
-    <row r="174" ht="20" customHeight="1">
-      <c r="A174" s="27" t="inlineStr">
+    <row r="175" ht="20" customHeight="1">
+      <c r="A175" s="27" t="inlineStr">
         <is>
           <t>第24条　月中に入社または退職した者についても、出勤日数に応じて日割り計算で支給する。</t>
         </is>
       </c>
     </row>
-    <row r="175" ht="8" customHeight="1"/>
-    <row r="176" ht="20" customHeight="1">
-      <c r="A176" s="26" t="inlineStr">
+    <row r="176" ht="8" customHeight="1"/>
+    <row r="177" ht="20" customHeight="1">
+      <c r="A177" s="26" t="inlineStr">
         <is>
           <t>（休職・休暇・在宅勤務時の取扱い）</t>
         </is>
       </c>
     </row>
-    <row r="177" ht="32" customHeight="1">
-      <c r="A177" s="27" t="inlineStr">
+    <row r="178" ht="32" customHeight="1">
+      <c r="A178" s="27" t="inlineStr">
         <is>
           <t>第25条　休職中・休暇中・休業中または在宅勤務の場合、通勤手当及び特別通勤手当は支給しない。</t>
         </is>
       </c>
     </row>
-    <row r="178" ht="8" customHeight="1"/>
-    <row r="179" ht="20" customHeight="1">
-      <c r="A179" s="26" t="inlineStr">
+    <row r="179" ht="8" customHeight="1"/>
+    <row r="180" ht="20" customHeight="1">
+      <c r="A180" s="26" t="inlineStr">
         <is>
           <t>（虚偽申請の禁止）</t>
         </is>
       </c>
     </row>
-    <row r="180" ht="32" customHeight="1">
-      <c r="A180" s="27" t="inlineStr">
+    <row r="181" ht="32" customHeight="1">
+      <c r="A181" s="27" t="inlineStr">
         <is>
           <t>第26条　通勤手当、特別通勤手当、住宅手当その他各種手当の申請に虚偽が発覚した場合、会社は入社時に遡って再計算を行い、超過支給分を返還請求できるものとする。</t>
         </is>
       </c>
     </row>
-    <row r="181" ht="8" customHeight="1"/>
-    <row r="182" ht="8" customHeight="1">
-      <c r="A182" s="28" t="inlineStr"/>
-      <c r="B182" s="12" t="n"/>
-      <c r="C182" s="12" t="n"/>
-      <c r="D182" s="12" t="n"/>
-      <c r="E182" s="12" t="n"/>
-    </row>
-    <row r="183" ht="10" customHeight="1"/>
-    <row r="184" ht="30" customHeight="1">
-      <c r="A184" s="25" t="inlineStr">
+    <row r="182" ht="8" customHeight="1"/>
+    <row r="183" ht="8" customHeight="1">
+      <c r="A183" s="28" t="inlineStr"/>
+      <c r="B183" s="12" t="n"/>
+      <c r="C183" s="12" t="n"/>
+      <c r="D183" s="12" t="n"/>
+      <c r="E183" s="12" t="n"/>
+    </row>
+    <row r="184" ht="10" customHeight="1"/>
+    <row r="185" ht="30" customHeight="1">
+      <c r="A185" s="25" t="inlineStr">
         <is>
           <t>第11章　雑則</t>
         </is>
       </c>
     </row>
-    <row r="185" ht="20" customHeight="1">
-      <c r="A185" s="26" t="inlineStr">
+    <row r="186" ht="20" customHeight="1">
+      <c r="A186" s="26" t="inlineStr">
         <is>
           <t>（周知）</t>
         </is>
       </c>
     </row>
-    <row r="186" ht="32" customHeight="1">
-      <c r="A186" s="27" t="inlineStr">
+    <row r="187" ht="32" customHeight="1">
+      <c r="A187" s="27" t="inlineStr">
         <is>
           <t>第27条　会社は、本規程の内容を従業員に周知し、常時確認できるよう掲示またはイントラネット等で公開する。</t>
         </is>
       </c>
     </row>
-    <row r="187" ht="8" customHeight="1"/>
-    <row r="188" ht="8" customHeight="1">
-      <c r="A188" s="28" t="inlineStr"/>
-      <c r="B188" s="12" t="n"/>
-      <c r="C188" s="12" t="n"/>
-      <c r="D188" s="12" t="n"/>
-      <c r="E188" s="12" t="n"/>
-    </row>
-    <row r="189" ht="10" customHeight="1"/>
-    <row r="190" ht="30" customHeight="1">
-      <c r="A190" s="25" t="inlineStr">
+    <row r="188" ht="8" customHeight="1"/>
+    <row r="189" ht="8" customHeight="1">
+      <c r="A189" s="28" t="inlineStr"/>
+      <c r="B189" s="12" t="n"/>
+      <c r="C189" s="12" t="n"/>
+      <c r="D189" s="12" t="n"/>
+      <c r="E189" s="12" t="n"/>
+    </row>
+    <row r="190" ht="10" customHeight="1"/>
+    <row r="191" ht="30" customHeight="1">
+      <c r="A191" s="25" t="inlineStr">
         <is>
           <t>附則</t>
-        </is>
-      </c>
-    </row>
-    <row r="191" ht="20" customHeight="1">
-      <c r="A191" s="27" t="inlineStr">
-        <is>
-          <t>1　本規程に定めのない事項は、就業規則その他関係規程による。</t>
         </is>
       </c>
     </row>
     <row r="192" ht="20" customHeight="1">
       <c r="A192" s="27" t="inlineStr">
         <is>
+          <t>1　本規程に定めのない事項は、就業規則その他関係規程による。</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="20" customHeight="1">
+      <c r="A193" s="27" t="inlineStr">
+        <is>
           <t>2　本規程は、令和8年2月1日から施行する。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="121">
+  <mergeCells count="122">
+    <mergeCell ref="A166:E166"/>
     <mergeCell ref="A48:E48"/>
     <mergeCell ref="A142:E142"/>
-    <mergeCell ref="A182:E182"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A168:E168"/>
     <mergeCell ref="A87:E87"/>
     <mergeCell ref="A128:E128"/>
+    <mergeCell ref="A193:E193"/>
+    <mergeCell ref="A137:E137"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="A46:E46"/>
     <mergeCell ref="A89:E89"/>
@@ -4628,10 +4623,9 @@
     <mergeCell ref="A57:E57"/>
     <mergeCell ref="A113:E113"/>
     <mergeCell ref="A139:E139"/>
-    <mergeCell ref="A179:E179"/>
     <mergeCell ref="A71:E71"/>
     <mergeCell ref="A185:E185"/>
-    <mergeCell ref="A184:E184"/>
+    <mergeCell ref="A181:E181"/>
     <mergeCell ref="A131:E131"/>
     <mergeCell ref="A100:E100"/>
     <mergeCell ref="A43:E43"/>
@@ -4642,29 +4636,31 @@
     <mergeCell ref="A115:E115"/>
     <mergeCell ref="A155:E155"/>
     <mergeCell ref="A93:E93"/>
-    <mergeCell ref="A173:E173"/>
     <mergeCell ref="A130:E130"/>
     <mergeCell ref="A77:E77"/>
     <mergeCell ref="A34:E34"/>
     <mergeCell ref="A83:E83"/>
     <mergeCell ref="A148:E148"/>
-    <mergeCell ref="A138:E138"/>
+    <mergeCell ref="A157:E157"/>
     <mergeCell ref="A132:E132"/>
     <mergeCell ref="A36:E36"/>
     <mergeCell ref="A69:E69"/>
     <mergeCell ref="A78:E78"/>
+    <mergeCell ref="A183:E183"/>
     <mergeCell ref="A118:E118"/>
+    <mergeCell ref="A133:E133"/>
     <mergeCell ref="A80:E80"/>
     <mergeCell ref="A120:E120"/>
     <mergeCell ref="A55:E55"/>
     <mergeCell ref="A95:E95"/>
     <mergeCell ref="A104:E104"/>
+    <mergeCell ref="A175:E175"/>
     <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A159:E159"/>
     <mergeCell ref="A97:E97"/>
     <mergeCell ref="A106:E106"/>
     <mergeCell ref="A81:E81"/>
     <mergeCell ref="A38:E38"/>
-    <mergeCell ref="A147:E147"/>
     <mergeCell ref="A161:E161"/>
     <mergeCell ref="A170:E170"/>
     <mergeCell ref="A31:E31"/>
@@ -4674,59 +4670,56 @@
     <mergeCell ref="A73:E73"/>
     <mergeCell ref="A123:E123"/>
     <mergeCell ref="A110:E110"/>
+    <mergeCell ref="A146:E146"/>
+    <mergeCell ref="A172:E172"/>
+    <mergeCell ref="A187:E187"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A174:E174"/>
     <mergeCell ref="A108:E108"/>
     <mergeCell ref="A149:E149"/>
-    <mergeCell ref="A158:E158"/>
+    <mergeCell ref="A189:E189"/>
     <mergeCell ref="A50:E50"/>
     <mergeCell ref="A86:E86"/>
     <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A151:E151"/>
     <mergeCell ref="A47:E47"/>
-    <mergeCell ref="A160:E160"/>
     <mergeCell ref="A141:E141"/>
     <mergeCell ref="A135:E135"/>
     <mergeCell ref="A150:E150"/>
+    <mergeCell ref="A144:E144"/>
     <mergeCell ref="A122:E122"/>
     <mergeCell ref="A125:E125"/>
-    <mergeCell ref="A134:E134"/>
     <mergeCell ref="A28:E28"/>
     <mergeCell ref="A112:E112"/>
-    <mergeCell ref="A152:E152"/>
     <mergeCell ref="A121:E121"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A44:E44"/>
-    <mergeCell ref="A167:E167"/>
-    <mergeCell ref="A176:E176"/>
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A114:E114"/>
     <mergeCell ref="A59:E59"/>
     <mergeCell ref="A98:E98"/>
     <mergeCell ref="A191:E191"/>
-    <mergeCell ref="A169:E169"/>
     <mergeCell ref="A51:E51"/>
+    <mergeCell ref="A178:E178"/>
     <mergeCell ref="A88:E88"/>
     <mergeCell ref="A70:E70"/>
+    <mergeCell ref="A153:E153"/>
     <mergeCell ref="A162:E162"/>
     <mergeCell ref="A54:E54"/>
     <mergeCell ref="A177:E177"/>
     <mergeCell ref="A90:E90"/>
     <mergeCell ref="A99:E99"/>
-    <mergeCell ref="A164:E164"/>
     <mergeCell ref="A74:E74"/>
-    <mergeCell ref="A145:E145"/>
     <mergeCell ref="A27:E27"/>
-    <mergeCell ref="A154:E154"/>
+    <mergeCell ref="A163:E163"/>
     <mergeCell ref="A101:E101"/>
     <mergeCell ref="A76:E76"/>
     <mergeCell ref="A85:E85"/>
-    <mergeCell ref="A188:E188"/>
     <mergeCell ref="A126:E126"/>
     <mergeCell ref="A140:E140"/>
     <mergeCell ref="A53:E53"/>
     <mergeCell ref="A109:E109"/>
     <mergeCell ref="A180:E180"/>
-    <mergeCell ref="A190:E190"/>
     <mergeCell ref="A102:E102"/>
     <mergeCell ref="A117:E117"/>
     <mergeCell ref="A111:E111"/>
@@ -5167,7 +5160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E106"/>
+  <dimension ref="A1:E137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -5292,69 +5285,75 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="20" customHeight="1">
+    <row r="38" ht="32" customHeight="1">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>3　「子の看護休暇」：小学校就学前の子の看護のために取得できる休暇をいう。</t>
+          <t>3　「子の看護等休暇」：小学校第3学年修了までの子の看護、予防接種・健康診断、感染症に伴う学級閉鎖等、入園（入学）式・卒園式への出席のために取得できる休暇をいう。</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="27" t="inlineStr">
         <is>
+          <t>5　「出生時育児休業」：子の出生後8週間以内に4週間（28日）まで取得できる休業をいう。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="27" t="inlineStr">
+        <is>
           <t>4　「介護休暇」：要介護状態にある家族の介護や通院付添のために取得できる休暇をいう。</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="8" customHeight="1"/>
-    <row r="41" ht="8" customHeight="1">
-      <c r="A41" s="28" t="inlineStr"/>
-      <c r="B41" s="12" t="n"/>
-      <c r="C41" s="12" t="n"/>
-      <c r="D41" s="12" t="n"/>
-      <c r="E41" s="12" t="n"/>
-    </row>
-    <row r="42" ht="10" customHeight="1"/>
-    <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="25" t="inlineStr">
+    <row r="41" ht="8" customHeight="1"/>
+    <row r="42" ht="8" customHeight="1">
+      <c r="A42" s="28" t="inlineStr"/>
+      <c r="B42" s="12" t="n"/>
+      <c r="C42" s="12" t="n"/>
+      <c r="D42" s="12" t="n"/>
+      <c r="E42" s="12" t="n"/>
+    </row>
+    <row r="43" ht="10" customHeight="1"/>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="25" t="inlineStr">
         <is>
           <t>第2章　育児休業</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="26" t="inlineStr">
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="26" t="inlineStr">
         <is>
           <t>（育児休業の取得要件）</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="32" customHeight="1">
-      <c r="A45" s="27" t="inlineStr">
+    <row r="46" ht="32" customHeight="1">
+      <c r="A46" s="27" t="inlineStr">
         <is>
           <t>第4条　従業員は、1歳に満たない子を養育する場合、会社に申し出ることにより育児休業を取得できる。</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="27" t="inlineStr">
-        <is>
-          <t>2　配偶者が常態として子を養育できる場合等、法令で育児休業が認められない場合は除く。</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="8" customHeight="1"/>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="26" t="inlineStr">
-        <is>
-          <t>（育児休業の期間）</t>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="27" t="inlineStr">
+        <is>
+          <t>2　育児休業は、子1人につき原則2回まで分割して取得できる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="48" customHeight="1">
+      <c r="A48" s="27" t="inlineStr">
+        <is>
+          <t>3　労使協定により、次の者を育児休業の対象から除外することがある。（1）継続雇用期間が1年未満の者　（2）申出の日から1年以内に雇用関係が終了することが明らかな者　（3）1週間の所定労働日数が2日以下の者</t>
         </is>
       </c>
     </row>
     <row r="49" ht="32" customHeight="1">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>第5条　育児休業の期間は、原則として子が1歳に達するまでとする。ただし、保育所に入所できない場合等、法令の定めに従い1歳6か月、最長2歳まで延長できる。</t>
+          <t>4　有期雇用の従業員は、子が1歳6か月に達する日までに労働契約が満了し更新されないことが明らかでない場合に取得できる。</t>
         </is>
       </c>
     </row>
@@ -5362,14 +5361,14 @@
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>（育児休業の申出）</t>
+          <t>（育児休業の期間）</t>
         </is>
       </c>
     </row>
     <row r="52" ht="32" customHeight="1">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>第6条　育児休業を取得しようとする従業員は、原則として休業開始予定日の1か月前までに、所定の書式により会社へ申し出なければならない。</t>
+          <t>第5条　育児休業の期間は、原則として子が1歳に達するまでとする。ただし、保育所に入所できない場合等、法令の定めに従い1歳6か月、最長2歳まで延長できる。</t>
         </is>
       </c>
     </row>
@@ -5377,341 +5376,527 @@
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="26" t="inlineStr">
         <is>
-          <t>（育児休業中の処遇）</t>
+          <t>（育児休業の申出）</t>
         </is>
       </c>
     </row>
     <row r="55" ht="32" customHeight="1">
       <c r="A55" s="27" t="inlineStr">
         <is>
-          <t>第7条　育児休業中は無給とする。ただし、雇用保険法に基づき育児休業給付金の受給が可能である。</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="27" t="inlineStr">
-        <is>
-          <t>2　社会保険料の免除については、健康保険法及び厚生年金保険法の定めに従う。</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="8" customHeight="1"/>
-    <row r="58" ht="8" customHeight="1">
-      <c r="A58" s="28" t="inlineStr"/>
-      <c r="B58" s="12" t="n"/>
-      <c r="C58" s="12" t="n"/>
-      <c r="D58" s="12" t="n"/>
-      <c r="E58" s="12" t="n"/>
-    </row>
-    <row r="59" ht="10" customHeight="1"/>
-    <row r="60" ht="30" customHeight="1">
-      <c r="A60" s="25" t="inlineStr">
-        <is>
-          <t>第3章　介護休業</t>
-        </is>
-      </c>
-    </row>
+          <t>第6条　育児休業を取得しようとする従業員は、原則として休業開始予定日の1か月前までに、所定の書式により会社へ申し出なければならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="8" customHeight="1"/>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="26" t="inlineStr">
+        <is>
+          <t>（出生時育児休業）</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="32" customHeight="1">
+      <c r="A58" s="27" t="inlineStr">
+        <is>
+          <t>第6条の2　従業員は、子の出生後8週間以内に、4週間（28日）を限度として、2回まで分割して出生時育児休業を取得できる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="32" customHeight="1">
+      <c r="A59" s="27" t="inlineStr">
+        <is>
+          <t>2　出生時育児休業を取得しようとする従業員は、原則として休業開始予定日の2週間前までに会社へ申し出なければならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="8" customHeight="1"/>
     <row r="61" ht="20" customHeight="1">
       <c r="A61" s="26" t="inlineStr">
         <is>
-          <t>（介護休業の取得要件）</t>
+          <t>（育児休業中の処遇）</t>
         </is>
       </c>
     </row>
     <row r="62" ht="32" customHeight="1">
       <c r="A62" s="27" t="inlineStr">
         <is>
+          <t>第7条　育児休業中は無給とする。ただし、雇用保険法に基づき育児休業給付金の受給が可能である。</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="27" t="inlineStr">
+        <is>
+          <t>2　社会保険料の免除については、健康保険法及び厚生年金保険法の定めに従う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="8" customHeight="1"/>
+    <row r="65" ht="8" customHeight="1">
+      <c r="A65" s="28" t="inlineStr"/>
+      <c r="B65" s="12" t="n"/>
+      <c r="C65" s="12" t="n"/>
+      <c r="D65" s="12" t="n"/>
+      <c r="E65" s="12" t="n"/>
+    </row>
+    <row r="66" ht="10" customHeight="1"/>
+    <row r="67" ht="30" customHeight="1">
+      <c r="A67" s="25" t="inlineStr">
+        <is>
+          <t>第3章　介護休業</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="20" customHeight="1">
+      <c r="A68" s="26" t="inlineStr">
+        <is>
+          <t>（介護休業の取得要件）</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="32" customHeight="1">
+      <c r="A69" s="27" t="inlineStr">
+        <is>
           <t>第8条　従業員は、要介護状態にある家族を介護する場合、会社に申し出ることにより介護休業を取得できる。</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="8" customHeight="1"/>
-    <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="26" t="inlineStr">
+    <row r="70" ht="8" customHeight="1"/>
+    <row r="71" ht="20" customHeight="1">
+      <c r="A71" s="26" t="inlineStr">
         <is>
           <t>（介護休業の期間）</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="32" customHeight="1">
-      <c r="A65" s="27" t="inlineStr">
+    <row r="72" ht="32" customHeight="1">
+      <c r="A72" s="27" t="inlineStr">
         <is>
           <t>第9条　介護休業は、対象家族1人につき通算93日まで取得できる。分割して3回まで分けて取得することができる。</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="8" customHeight="1"/>
-    <row r="67" ht="20" customHeight="1">
-      <c r="A67" s="26" t="inlineStr">
+    <row r="73" ht="8" customHeight="1"/>
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="26" t="inlineStr">
         <is>
           <t>（介護休業の申出）</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="32" customHeight="1">
-      <c r="A68" s="27" t="inlineStr">
+    <row r="75" ht="32" customHeight="1">
+      <c r="A75" s="27" t="inlineStr">
         <is>
           <t>第10条　介護休業を取得しようとする従業員は、原則として休業開始予定日の2週間前までに、所定の書式により会社へ申し出なければならない。</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="8" customHeight="1"/>
-    <row r="70" ht="20" customHeight="1">
-      <c r="A70" s="26" t="inlineStr">
+    <row r="76" ht="8" customHeight="1"/>
+    <row r="77" ht="20" customHeight="1">
+      <c r="A77" s="26" t="inlineStr">
         <is>
           <t>（介護休業中の処遇）</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="32" customHeight="1">
-      <c r="A71" s="27" t="inlineStr">
+    <row r="78" ht="32" customHeight="1">
+      <c r="A78" s="27" t="inlineStr">
         <is>
           <t>第11条　介護休業中は無給とする。ただし、雇用保険法に基づき介護休業給付金の受給が可能である。</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="8" customHeight="1"/>
-    <row r="73" ht="8" customHeight="1">
-      <c r="A73" s="28" t="inlineStr"/>
-      <c r="B73" s="12" t="n"/>
-      <c r="C73" s="12" t="n"/>
-      <c r="D73" s="12" t="n"/>
-      <c r="E73" s="12" t="n"/>
-    </row>
-    <row r="74" ht="10" customHeight="1"/>
-    <row r="75" ht="30" customHeight="1">
-      <c r="A75" s="25" t="inlineStr">
-        <is>
-          <t>第4章　子の看護休暇・介護休暇</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="20" customHeight="1">
-      <c r="A76" s="26" t="inlineStr">
-        <is>
-          <t>（子の看護休暇）</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="32" customHeight="1">
-      <c r="A77" s="27" t="inlineStr">
-        <is>
-          <t>第12条　従業員は、小学校就学前の子が病気やけがをした場合、看護のため年5日（子が2人以上の場合は年10日）を限度として休暇を取得できる。</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="20" customHeight="1">
-      <c r="A78" s="27" t="inlineStr">
-        <is>
-          <t>2　子の看護休暇は、1日または半日単位で取得できる。</t>
-        </is>
-      </c>
-    </row>
     <row r="79" ht="8" customHeight="1"/>
-    <row r="80" ht="20" customHeight="1">
-      <c r="A80" s="26" t="inlineStr">
-        <is>
-          <t>（介護休暇）</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="32" customHeight="1">
-      <c r="A81" s="27" t="inlineStr">
-        <is>
-          <t>第13条　従業員は、要介護状態にある家族の介護や通院付添のため、年5日（対象家族が2人以上の場合は年10日）を限度として休暇を取得できる。</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="20" customHeight="1">
-      <c r="A82" s="27" t="inlineStr">
-        <is>
-          <t>2　介護休暇は、1日または半日単位で取得できる。</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="8" customHeight="1"/>
-    <row r="84" ht="8" customHeight="1">
-      <c r="A84" s="28" t="inlineStr"/>
-      <c r="B84" s="12" t="n"/>
-      <c r="C84" s="12" t="n"/>
-      <c r="D84" s="12" t="n"/>
-      <c r="E84" s="12" t="n"/>
-    </row>
-    <row r="85" ht="10" customHeight="1"/>
-    <row r="86" ht="30" customHeight="1">
-      <c r="A86" s="25" t="inlineStr">
-        <is>
-          <t>第5章　復職・不利益取扱い禁止</t>
-        </is>
-      </c>
-    </row>
+    <row r="80" ht="8" customHeight="1">
+      <c r="A80" s="28" t="inlineStr"/>
+      <c r="B80" s="12" t="n"/>
+      <c r="C80" s="12" t="n"/>
+      <c r="D80" s="12" t="n"/>
+      <c r="E80" s="12" t="n"/>
+    </row>
+    <row r="81" ht="10" customHeight="1"/>
+    <row r="82" ht="30" customHeight="1">
+      <c r="A82" s="25" t="inlineStr">
+        <is>
+          <t>第4章　子の看護等休暇・介護休暇</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="26" t="inlineStr">
+        <is>
+          <t>（子の看護等休暇）</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="48" customHeight="1">
+      <c r="A84" s="27" t="inlineStr">
+        <is>
+          <t>第12条　従業員は、小学校第3学年修了までの子の看護、予防接種・健康診断、感染症に伴う学級閉鎖等、入園（入学）式・卒園式への出席のため、年5日（子が2人以上の場合は年10日）を限度として休暇を取得できる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="20" customHeight="1">
+      <c r="A85" s="27" t="inlineStr">
+        <is>
+          <t>2　子の看護等休暇は、1日または時間単位で取得できる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="8" customHeight="1"/>
     <row r="87" ht="20" customHeight="1">
       <c r="A87" s="26" t="inlineStr">
         <is>
-          <t>（復職）</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="48" customHeight="1">
+          <t>（介護休暇）</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="32" customHeight="1">
       <c r="A88" s="27" t="inlineStr">
         <is>
-          <t>第14条　育児休業または介護休業を終了した従業員は、原則として休業前と同じ職務に復職させる。ただし、業務運営上やむを得ない場合は、同等の地位・待遇を有する職務に配置することができる。</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="8" customHeight="1"/>
-    <row r="90" ht="20" customHeight="1">
-      <c r="A90" s="26" t="inlineStr">
-        <is>
-          <t>（不利益取扱い禁止）</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="32" customHeight="1">
-      <c r="A91" s="27" t="inlineStr">
-        <is>
-          <t>第15条　会社は、従業員が育児休業・介護休業・子の看護休暇・介護休暇を取得したことを理由として、解雇その他不利益な取扱いをしてはならない。</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="8" customHeight="1"/>
-    <row r="93" ht="8" customHeight="1">
-      <c r="A93" s="28" t="inlineStr"/>
-      <c r="B93" s="12" t="n"/>
-      <c r="C93" s="12" t="n"/>
-      <c r="D93" s="12" t="n"/>
-      <c r="E93" s="12" t="n"/>
-    </row>
-    <row r="94" ht="10" customHeight="1"/>
-    <row r="95" ht="30" customHeight="1">
-      <c r="A95" s="25" t="inlineStr">
-        <is>
-          <t>第6章　雑則</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="20" customHeight="1">
-      <c r="A96" s="26" t="inlineStr">
-        <is>
-          <t>（制度の周知）</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="32" customHeight="1">
-      <c r="A97" s="27" t="inlineStr">
-        <is>
-          <t>第16条　会社は、本規程の内容を就業規則とともに従業員へ周知し、希望者が適切に制度を利用できるよう努めなければならない。</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="8" customHeight="1"/>
-    <row r="99" ht="20" customHeight="1">
-      <c r="A99" s="26" t="inlineStr">
-        <is>
-          <t>（個人情報保護）</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="32" customHeight="1">
-      <c r="A100" s="27" t="inlineStr">
-        <is>
-          <t>第17条　会社は、休業申請や取得に関して知り得た個人情報を適切に管理し、業務遂行上必要な場合を除き、第三者に開示してはならない。</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="8" customHeight="1"/>
-    <row r="102" ht="8" customHeight="1">
-      <c r="A102" s="28" t="inlineStr"/>
-      <c r="B102" s="12" t="n"/>
-      <c r="C102" s="12" t="n"/>
-      <c r="D102" s="12" t="n"/>
-      <c r="E102" s="12" t="n"/>
-    </row>
-    <row r="103" ht="10" customHeight="1"/>
-    <row r="104" ht="30" customHeight="1">
-      <c r="A104" s="25" t="inlineStr">
-        <is>
-          <t>附則</t>
+          <t>第13条　従業員は、要介護状態にある家族の介護や通院付添のため、年5日（対象家族が2人以上の場合は年10日）を限度として休暇を取得できる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="27" t="inlineStr">
+        <is>
+          <t>2　介護休暇は、1日または時間単位で取得できる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="8" customHeight="1"/>
+    <row r="91" ht="8" customHeight="1">
+      <c r="A91" s="28" t="inlineStr"/>
+      <c r="B91" s="12" t="n"/>
+      <c r="C91" s="12" t="n"/>
+      <c r="D91" s="12" t="n"/>
+      <c r="E91" s="12" t="n"/>
+    </row>
+    <row r="92" ht="10" customHeight="1"/>
+    <row r="93" ht="30" customHeight="1">
+      <c r="A93" s="25" t="inlineStr">
+        <is>
+          <t>第4章の2　働き方の制限・措置</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="26" t="inlineStr">
+        <is>
+          <t>（所定外労働の制限）</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="32" customHeight="1">
+      <c r="A95" s="27" t="inlineStr">
+        <is>
+          <t>第13条の2　小学校就学前の子を養育する従業員、または要介護状態にある家族を介護する従業員が請求した場合、事業の正常な運営を妨げる場合を除き、所定労働時間を超えて労働させない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="8" customHeight="1"/>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="26" t="inlineStr">
+        <is>
+          <t>（時間外労働・深夜業の制限）</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="48" customHeight="1">
+      <c r="A98" s="27" t="inlineStr">
+        <is>
+          <t>第13条の3　前条の従業員が請求した場合、時間外労働は1か月24時間、1年150時間を超えないものとし、深夜（午後10時から午前5時まで）に労働させない。ただし、法令に定める除外者はこの限りでない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="8" customHeight="1"/>
+    <row r="100" ht="20" customHeight="1">
+      <c r="A100" s="26" t="inlineStr">
+        <is>
+          <t>（短時間勤務）</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="32" customHeight="1">
+      <c r="A101" s="27" t="inlineStr">
+        <is>
+          <t>第13条の4　3歳に満たない子を養育する従業員、または要介護状態にある家族を介護する従業員は、申し出により、所定労働時間を1日6時間とする短時間勤務を利用できる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="8" customHeight="1"/>
+    <row r="103" ht="20" customHeight="1">
+      <c r="A103" s="26" t="inlineStr">
+        <is>
+          <t>（柔軟な働き方を実現するための措置）</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="32" customHeight="1">
+      <c r="A104" s="27" t="inlineStr">
+        <is>
+          <t>第13条の5　3歳から小学校就学前の子を養育する従業員に対し、会社は次の措置を講じ、従業員はいずれか1つを選択して利用できる。</t>
         </is>
       </c>
     </row>
     <row r="105" ht="20" customHeight="1">
       <c r="A105" s="27" t="inlineStr">
         <is>
-          <t>1　本規程に定めのない事項は、育児・介護休業法、就業規則その他関係規程による。</t>
+          <t>1　始業・終業時刻の変更（時差出勤）</t>
         </is>
       </c>
     </row>
     <row r="106" ht="20" customHeight="1">
       <c r="A106" s="27" t="inlineStr">
         <is>
+          <t>2　養育両立支援休暇（年10日、時間単位で取得可）</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="8" customHeight="1"/>
+    <row r="108" ht="20" customHeight="1">
+      <c r="A108" s="26" t="inlineStr">
+        <is>
+          <t>（個別周知・意向確認）</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="32" customHeight="1">
+      <c r="A109" s="27" t="inlineStr">
+        <is>
+          <t>第13条の6　会社は、従業員から本人または配偶者の妊娠・出産の申出があったとき、及び子が3歳になる前の適切な時期に、育児休業等の制度を個別に周知し、取得や働き方の意向を確認する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="32" customHeight="1">
+      <c r="A110" s="27" t="inlineStr">
+        <is>
+          <t>2　会社は、従業員から家族の介護に直面した旨の申出があったとき、介護休業等の制度を個別に周知し、意向を確認する。また、40歳に達した従業員に対し、介護両立支援制度の情報を提供する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="8" customHeight="1"/>
+    <row r="112" ht="20" customHeight="1">
+      <c r="A112" s="26" t="inlineStr">
+        <is>
+          <t>（ハラスメントの防止）</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="32" customHeight="1">
+      <c r="A113" s="27" t="inlineStr">
+        <is>
+          <t>第13条の7　会社は、妊娠・出産、育児休業・介護休業等の利用に関する言動により従業員の就業環境が害されることのないよう、相談体制の整備その他必要な措置を講じる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="8" customHeight="1"/>
+    <row r="115" ht="8" customHeight="1">
+      <c r="A115" s="28" t="inlineStr"/>
+      <c r="B115" s="12" t="n"/>
+      <c r="C115" s="12" t="n"/>
+      <c r="D115" s="12" t="n"/>
+      <c r="E115" s="12" t="n"/>
+    </row>
+    <row r="116" ht="10" customHeight="1"/>
+    <row r="117" ht="30" customHeight="1">
+      <c r="A117" s="25" t="inlineStr">
+        <is>
+          <t>第5章　復職・不利益取扱い禁止</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="20" customHeight="1">
+      <c r="A118" s="26" t="inlineStr">
+        <is>
+          <t>（復職）</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="48" customHeight="1">
+      <c r="A119" s="27" t="inlineStr">
+        <is>
+          <t>第14条　育児休業または介護休業を終了した従業員は、原則として休業前と同じ職務に復職させる。ただし、業務運営上やむを得ない場合は、同等の地位・待遇を有する職務に配置することができる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="8" customHeight="1"/>
+    <row r="121" ht="20" customHeight="1">
+      <c r="A121" s="26" t="inlineStr">
+        <is>
+          <t>（不利益取扱い禁止）</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="32" customHeight="1">
+      <c r="A122" s="27" t="inlineStr">
+        <is>
+          <t>第15条　会社は、従業員が育児休業・出生時育児休業・介護休業・子の看護等休暇・介護休暇その他本規程の制度を利用したことを理由として、解雇その他不利益な取扱いをしてはならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="8" customHeight="1"/>
+    <row r="124" ht="8" customHeight="1">
+      <c r="A124" s="28" t="inlineStr"/>
+      <c r="B124" s="12" t="n"/>
+      <c r="C124" s="12" t="n"/>
+      <c r="D124" s="12" t="n"/>
+      <c r="E124" s="12" t="n"/>
+    </row>
+    <row r="125" ht="10" customHeight="1"/>
+    <row r="126" ht="30" customHeight="1">
+      <c r="A126" s="25" t="inlineStr">
+        <is>
+          <t>第6章　雑則</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="20" customHeight="1">
+      <c r="A127" s="26" t="inlineStr">
+        <is>
+          <t>（制度の周知）</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="32" customHeight="1">
+      <c r="A128" s="27" t="inlineStr">
+        <is>
+          <t>第16条　会社は、本規程の内容を就業規則とともに従業員へ周知し、希望者が適切に制度を利用できるよう努めなければならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="8" customHeight="1"/>
+    <row r="130" ht="20" customHeight="1">
+      <c r="A130" s="26" t="inlineStr">
+        <is>
+          <t>（個人情報保護）</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="32" customHeight="1">
+      <c r="A131" s="27" t="inlineStr">
+        <is>
+          <t>第17条　会社は、休業申請や取得に関して知り得た個人情報を適切に管理し、業務遂行上必要な場合を除き、第三者に開示してはならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="8" customHeight="1"/>
+    <row r="133" ht="8" customHeight="1">
+      <c r="A133" s="28" t="inlineStr"/>
+      <c r="B133" s="12" t="n"/>
+      <c r="C133" s="12" t="n"/>
+      <c r="D133" s="12" t="n"/>
+      <c r="E133" s="12" t="n"/>
+    </row>
+    <row r="134" ht="10" customHeight="1"/>
+    <row r="135" ht="30" customHeight="1">
+      <c r="A135" s="25" t="inlineStr">
+        <is>
+          <t>附則</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="20" customHeight="1">
+      <c r="A136" s="27" t="inlineStr">
+        <is>
+          <t>1　本規程に定めのない事項は、育児・介護休業法、就業規則その他関係規程による。</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="20" customHeight="1">
+      <c r="A137" s="27" t="inlineStr">
+        <is>
           <t>2　本規程は、令和8年2月1日から施行する。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="61">
-    <mergeCell ref="A30:E30"/>
+  <mergeCells count="84">
     <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A77:E77"/>
     <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A73:E73"/>
-    <mergeCell ref="A64:E64"/>
-    <mergeCell ref="A82:E82"/>
-    <mergeCell ref="A60:E60"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="A51:E51"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A45:E45"/>
-    <mergeCell ref="A36:E36"/>
-    <mergeCell ref="A61:E61"/>
-    <mergeCell ref="A88:E88"/>
-    <mergeCell ref="A70:E70"/>
+    <mergeCell ref="A94:E94"/>
+    <mergeCell ref="A103:E103"/>
     <mergeCell ref="A87:E87"/>
     <mergeCell ref="A65:E65"/>
-    <mergeCell ref="A78:E78"/>
-    <mergeCell ref="A54:E54"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A90:E90"/>
-    <mergeCell ref="A99:E99"/>
+    <mergeCell ref="A128:E128"/>
+    <mergeCell ref="A137:E137"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="A46:E46"/>
+    <mergeCell ref="A89:E89"/>
+    <mergeCell ref="A136:E136"/>
+    <mergeCell ref="A105:E105"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A57:E57"/>
+    <mergeCell ref="A113:E113"/>
+    <mergeCell ref="A71:E71"/>
+    <mergeCell ref="A91:E91"/>
+    <mergeCell ref="A131:E131"/>
+    <mergeCell ref="A100:E100"/>
+    <mergeCell ref="A52:E52"/>
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="A115:E115"/>
+    <mergeCell ref="A93:E93"/>
+    <mergeCell ref="A130:E130"/>
+    <mergeCell ref="A77:E77"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A83:E83"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A119:E119"/>
+    <mergeCell ref="A69:E69"/>
+    <mergeCell ref="A78:E78"/>
+    <mergeCell ref="A118:E118"/>
     <mergeCell ref="A75:E75"/>
-    <mergeCell ref="A84:E84"/>
+    <mergeCell ref="A133:E133"/>
     <mergeCell ref="A80:E80"/>
-    <mergeCell ref="A56:E56"/>
-    <mergeCell ref="A27:E27"/>
-    <mergeCell ref="A105:E105"/>
     <mergeCell ref="A55:E55"/>
-    <mergeCell ref="A26:E26"/>
     <mergeCell ref="A95:E95"/>
-    <mergeCell ref="A86:E86"/>
     <mergeCell ref="A104:E104"/>
-    <mergeCell ref="A76:E76"/>
-    <mergeCell ref="A71:E71"/>
     <mergeCell ref="A32:E32"/>
     <mergeCell ref="A97:E97"/>
     <mergeCell ref="A106:E106"/>
-    <mergeCell ref="A91:E91"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A67:E67"/>
+    <mergeCell ref="A82:E82"/>
+    <mergeCell ref="A110:E110"/>
+    <mergeCell ref="A124:E124"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A108:E108"/>
+    <mergeCell ref="A84:E84"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A135:E135"/>
+    <mergeCell ref="A122:E122"/>
+    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A112:E112"/>
+    <mergeCell ref="A121:E121"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A127:E127"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A59:E59"/>
+    <mergeCell ref="A98:E98"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="A61:E61"/>
+    <mergeCell ref="A88:E88"/>
+    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A74:E74"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A101:E101"/>
+    <mergeCell ref="A85:E85"/>
+    <mergeCell ref="A126:E126"/>
+    <mergeCell ref="A109:E109"/>
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A62:E62"/>
-    <mergeCell ref="A43:E43"/>
-    <mergeCell ref="A38:E38"/>
-    <mergeCell ref="A81:E81"/>
-    <mergeCell ref="A96:E96"/>
-    <mergeCell ref="A52:E52"/>
-    <mergeCell ref="A100:E100"/>
-    <mergeCell ref="A28:E28"/>
     <mergeCell ref="A68:E68"/>
-    <mergeCell ref="A102:E102"/>
-    <mergeCell ref="A93:E93"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A31:E31"/>
-    <mergeCell ref="A44:E44"/>
-    <mergeCell ref="A58:E58"/>
-    <mergeCell ref="A67:E67"/>
+    <mergeCell ref="A117:E117"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5736,7 +5921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E105"/>
+  <dimension ref="A1:E114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -5909,59 +6094,65 @@
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
-          <t>（退職の申出）</t>
+          <t>（定年）</t>
         </is>
       </c>
     </row>
     <row r="48" ht="32" customHeight="1">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>第5条　従業員が自己都合により退職を希望する場合は、原則として退職希望日の30日前までに所定の退職届を提出しなければならない。</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="8" customHeight="1"/>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="26" t="inlineStr">
-        <is>
-          <t>（引継ぎ義務）</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="32" customHeight="1">
-      <c r="A51" s="27" t="inlineStr">
-        <is>
-          <t>第6条　退職する従業員は、会社が指定する業務の引継ぎを誠実に行い、職務上の責任を果たさなければならない。</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="8" customHeight="1"/>
+          <t>第4条の2　従業員の定年は満60歳とし、満60歳に達した日の属する月の末日をもって退職とする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="32" customHeight="1">
+      <c r="A49" s="27" t="inlineStr">
+        <is>
+          <t>2　定年に達した従業員が希望する場合は、高年齢者雇用安定法に基づき、満65歳まで継続雇用する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="8" customHeight="1"/>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="26" t="inlineStr">
+        <is>
+          <t>（退職の申出）</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="32" customHeight="1">
+      <c r="A52" s="27" t="inlineStr">
+        <is>
+          <t>第5条　従業員が自己都合により退職を希望する場合は、円滑な引継ぎのため、原則として退職希望日の30日前までに所定の退職届を提出するよう努めなければならない。</t>
+        </is>
+      </c>
+    </row>
     <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="26" t="inlineStr">
-        <is>
-          <t>（会社物品の返還）</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="32" customHeight="1">
-      <c r="A54" s="27" t="inlineStr">
-        <is>
-          <t>第7条　退職する従業員は、退職日までに会社から貸与された備品、制服、身分証、書類、電子機器その他の物品を返還しなければならない。</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="8" customHeight="1"/>
-    <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="26" t="inlineStr">
-        <is>
-          <t>（退職証明書の交付）</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="32" customHeight="1">
+      <c r="A53" s="27" t="inlineStr">
+        <is>
+          <t>2　前項にかかわらず、退職の効力は民法の定めによる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="8" customHeight="1"/>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="26" t="inlineStr">
+        <is>
+          <t>（解雇予告）</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="48" customHeight="1">
+      <c r="A56" s="27" t="inlineStr">
+        <is>
+          <t>第5条の2　会社が従業員を解雇する場合は、少なくとも30日前に予告するか、30日分以上の平均賃金（解雇予告手当）を支払う。ただし、労働基準監督署長の認定を受けた場合はこの限りでない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>第8条　従業員が退職した場合、本人の請求に基づき、労働基準法第22条に定める退職証明書を交付する。</t>
+          <t>2　予告の日数は、平均賃金を支払った日数分短縮することができる。</t>
         </is>
       </c>
     </row>
@@ -5969,14 +6160,14 @@
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="26" t="inlineStr">
         <is>
-          <t>（賃金の精算）</t>
+          <t>（引継ぎ義務）</t>
         </is>
       </c>
     </row>
     <row r="60" ht="32" customHeight="1">
       <c r="A60" s="27" t="inlineStr">
         <is>
-          <t>第9条　退職に際しては、労働基準法第23条に基づき、未払賃金その他の金銭を退職日から7日以内に支払う。</t>
+          <t>第6条　退職する従業員は、会社が指定する業務の引継ぎを誠実に行い、職務上の責任を果たさなければならない。</t>
         </is>
       </c>
     </row>
@@ -5984,44 +6175,44 @@
     <row r="62" ht="20" customHeight="1">
       <c r="A62" s="26" t="inlineStr">
         <is>
-          <t>（秘密保持義務）</t>
+          <t>（会社物品の返還）</t>
         </is>
       </c>
     </row>
     <row r="63" ht="32" customHeight="1">
       <c r="A63" s="27" t="inlineStr">
         <is>
-          <t>第10条　退職した従業員は、在職中に知り得た会社の営業秘密、顧客情報、個人情報その他の秘密を退職後も漏洩してはならない。</t>
+          <t>第7条　退職する従業員は、退職日までに会社から貸与された備品、制服、身分証、書類、電子機器その他の物品を返還しなければならない。</t>
         </is>
       </c>
     </row>
     <row r="64" ht="8" customHeight="1"/>
-    <row r="65" ht="8" customHeight="1">
-      <c r="A65" s="28" t="inlineStr"/>
-      <c r="B65" s="12" t="n"/>
-      <c r="C65" s="12" t="n"/>
-      <c r="D65" s="12" t="n"/>
-      <c r="E65" s="12" t="n"/>
-    </row>
-    <row r="66" ht="10" customHeight="1"/>
-    <row r="67" ht="30" customHeight="1">
-      <c r="A67" s="25" t="inlineStr">
-        <is>
-          <t>第3章　退職金</t>
-        </is>
-      </c>
-    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="26" t="inlineStr">
+        <is>
+          <t>（退職証明書の交付）</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="32" customHeight="1">
+      <c r="A66" s="27" t="inlineStr">
+        <is>
+          <t>第8条　従業員が退職した場合、本人の請求に基づき、労働基準法第22条に定める退職証明書を交付する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="8" customHeight="1"/>
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="26" t="inlineStr">
         <is>
-          <t>（支給対象者）</t>
+          <t>（賃金の精算）</t>
         </is>
       </c>
     </row>
     <row r="69" ht="32" customHeight="1">
       <c r="A69" s="27" t="inlineStr">
         <is>
-          <t>第11条　勤続1年以上の従業員が退職した場合、会社は退職金を支給する。ただし、第15条に定める不支給事由に該当する場合は支給しない。</t>
+          <t>第9条　退職に際しては、労働基準法第23条に基づき、本人（死亡の場合は遺族）の請求があったときから7日以内に、未払賃金その他の金銭を支払う。</t>
         </is>
       </c>
     </row>
@@ -6029,341 +6220,393 @@
     <row r="71" ht="20" customHeight="1">
       <c r="A71" s="26" t="inlineStr">
         <is>
-          <t>（勤続年数の算定）</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="20" customHeight="1">
+          <t>（秘密保持義務）</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="32" customHeight="1">
       <c r="A72" s="27" t="inlineStr">
         <is>
-          <t>第12条　勤続年数は、入社日から退職日までの期間により算定する。</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="20" customHeight="1">
-      <c r="A73" s="27" t="inlineStr">
-        <is>
-          <t>2　1年未満の端数については次のとおりとする。</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="20" customHeight="1">
-      <c r="A74" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　1　6か月未満の端数は切り捨てる。</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　2　6か月以上の端数は1年に切り上げる。</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="8" customHeight="1"/>
+          <t>第10条　退職した従業員は、在職中に知り得た会社の営業秘密、顧客情報、個人情報その他の秘密を退職後も漏洩してはならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="8" customHeight="1"/>
+    <row r="74" ht="8" customHeight="1">
+      <c r="A74" s="28" t="inlineStr"/>
+      <c r="B74" s="12" t="n"/>
+      <c r="C74" s="12" t="n"/>
+      <c r="D74" s="12" t="n"/>
+      <c r="E74" s="12" t="n"/>
+    </row>
+    <row r="75" ht="10" customHeight="1"/>
+    <row r="76" ht="30" customHeight="1">
+      <c r="A76" s="25" t="inlineStr">
+        <is>
+          <t>第3章　退職金</t>
+        </is>
+      </c>
+    </row>
     <row r="77" ht="20" customHeight="1">
       <c r="A77" s="26" t="inlineStr">
         <is>
-          <t>（退職金の算定方法）</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="20" customHeight="1">
+          <t>（支給対象者）</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="32" customHeight="1">
       <c r="A78" s="27" t="inlineStr">
         <is>
-          <t>第13条　退職金の額は、次の算式により算定する。</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="20" customHeight="1">
-      <c r="A79" s="27" t="inlineStr">
-        <is>
-          <t>退職金 ＝ 退職時基本給 × 支給係数 × 勤続年数</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="8" customHeight="1"/>
+          <t>第11条　勤続1年以上の従業員が退職した場合、会社は退職金を支給する。ただし、第15条に定める不支給事由に該当する場合は支給しない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="8" customHeight="1"/>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="26" t="inlineStr">
+        <is>
+          <t>（勤続年数の算定）</t>
+        </is>
+      </c>
+    </row>
     <row r="81" ht="20" customHeight="1">
-      <c r="A81" s="26" t="inlineStr">
-        <is>
-          <t>（支給係数）</t>
+      <c r="A81" s="27" t="inlineStr">
+        <is>
+          <t>第12条　勤続年数は、入社日から退職日までの期間により算定する。</t>
         </is>
       </c>
     </row>
     <row r="82" ht="20" customHeight="1">
       <c r="A82" s="27" t="inlineStr">
         <is>
+          <t>2　1年未満の端数については次のとおりとする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　1　6か月未満の端数は切り捨てる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="20" customHeight="1">
+      <c r="A84" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　2　6か月以上の端数は1年に切り上げる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="8" customHeight="1"/>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="26" t="inlineStr">
+        <is>
+          <t>（退職金の算定方法）</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="27" t="inlineStr">
+        <is>
+          <t>第13条　退職金の額は、次の算式により算定する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="20" customHeight="1">
+      <c r="A88" s="27" t="inlineStr">
+        <is>
+          <t>退職金 ＝ 退職時基本給 × 支給係数 × 勤続年数</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="8" customHeight="1"/>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="26" t="inlineStr">
+        <is>
+          <t>（支給係数）</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="27" t="inlineStr">
+        <is>
           <t>第14条　支給係数は、勤続年数及び退職理由に応じて次のとおりとする。</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="20" customHeight="1">
-      <c r="A83" s="29" t="inlineStr">
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="29" t="inlineStr">
         <is>
           <t>勤続年数</t>
         </is>
       </c>
-      <c r="B83" s="33" t="inlineStr">
+      <c r="B92" s="33" t="inlineStr">
         <is>
           <t>自己都合</t>
         </is>
       </c>
-      <c r="C83" s="33" t="inlineStr">
+      <c r="C92" s="33" t="inlineStr">
         <is>
           <t>会社都合</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="20" customHeight="1">
-      <c r="A84" s="31" t="inlineStr">
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="31" t="inlineStr">
         <is>
           <t>1年以上3年未満</t>
         </is>
       </c>
-      <c r="B84" s="34" t="inlineStr">
+      <c r="B93" s="34" t="inlineStr">
         <is>
           <t>0.3</t>
         </is>
       </c>
-      <c r="C84" s="34" t="inlineStr">
+      <c r="C93" s="34" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="20" customHeight="1">
-      <c r="A85" s="31" t="inlineStr">
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="31" t="inlineStr">
         <is>
           <t>3年以上6年未満</t>
         </is>
       </c>
-      <c r="B85" s="34" t="inlineStr">
+      <c r="B94" s="34" t="inlineStr">
         <is>
           <t>0.4</t>
         </is>
       </c>
-      <c r="C85" s="34" t="inlineStr">
+      <c r="C94" s="34" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="20" customHeight="1">
-      <c r="A86" s="31" t="inlineStr">
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="31" t="inlineStr">
         <is>
           <t>6年以上9年未満</t>
         </is>
       </c>
-      <c r="B86" s="34" t="inlineStr">
+      <c r="B95" s="34" t="inlineStr">
         <is>
           <t>0.6</t>
         </is>
       </c>
-      <c r="C86" s="34" t="inlineStr">
+      <c r="C95" s="34" t="inlineStr">
         <is>
           <t>0.7</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="20" customHeight="1">
-      <c r="A87" s="31" t="inlineStr">
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="31" t="inlineStr">
         <is>
           <t>9年以上15年未満</t>
         </is>
       </c>
-      <c r="B87" s="34" t="inlineStr">
+      <c r="B96" s="34" t="inlineStr">
         <is>
           <t>0.7</t>
         </is>
       </c>
-      <c r="C87" s="34" t="inlineStr">
+      <c r="C96" s="34" t="inlineStr">
         <is>
           <t>0.8</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="20" customHeight="1">
-      <c r="A88" s="31" t="inlineStr">
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="31" t="inlineStr">
         <is>
           <t>15年以上25年未満</t>
         </is>
       </c>
-      <c r="B88" s="34" t="inlineStr">
+      <c r="B97" s="34" t="inlineStr">
         <is>
           <t>0.8</t>
         </is>
       </c>
-      <c r="C88" s="34" t="inlineStr">
+      <c r="C97" s="34" t="inlineStr">
         <is>
           <t>0.9</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="20" customHeight="1">
-      <c r="A89" s="31" t="inlineStr">
+    <row r="98" ht="20" customHeight="1">
+      <c r="A98" s="31" t="inlineStr">
         <is>
           <t>25年以上</t>
         </is>
       </c>
-      <c r="B89" s="34" t="inlineStr">
+      <c r="B98" s="34" t="inlineStr">
         <is>
           <t>0.9</t>
         </is>
       </c>
-      <c r="C89" s="34" t="inlineStr">
+      <c r="C98" s="34" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="8" customHeight="1"/>
-    <row r="91" ht="20" customHeight="1">
-      <c r="A91" s="26" t="inlineStr">
+    <row r="99" ht="8" customHeight="1"/>
+    <row r="100" ht="20" customHeight="1">
+      <c r="A100" s="26" t="inlineStr">
         <is>
           <t>（不支給事由）</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="20" customHeight="1">
-      <c r="A92" s="27" t="inlineStr">
+    <row r="101" ht="20" customHeight="1">
+      <c r="A101" s="27" t="inlineStr">
         <is>
           <t>第15条　従業員が次の各号のいずれかに該当する場合は、退職金を支給しない。</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="20" customHeight="1">
-      <c r="A93" s="27" t="inlineStr">
+    <row r="102" ht="20" customHeight="1">
+      <c r="A102" s="27" t="inlineStr">
         <is>
           <t>1　懲戒解雇された場合</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="20" customHeight="1">
-      <c r="A94" s="27" t="inlineStr">
+    <row r="103" ht="20" customHeight="1">
+      <c r="A103" s="27" t="inlineStr">
         <is>
           <t>2　重大な背信行為により会社に著しい損害を与えた場合</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="20" customHeight="1">
-      <c r="A95" s="27" t="inlineStr">
-        <is>
-          <t>3　虚偽の申告により雇用契約を締結したことが判明した場合</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="8" customHeight="1"/>
-    <row r="97" ht="20" customHeight="1">
-      <c r="A97" s="26" t="inlineStr">
-        <is>
-          <t>（支給手続）</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="20" customHeight="1">
-      <c r="A98" s="27" t="inlineStr">
-        <is>
-          <t>第16条　退職金は、退職日から2か月以内に本人の指定口座に振り込む。</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="20" customHeight="1">
-      <c r="A99" s="27" t="inlineStr">
-        <is>
-          <t>2　会社は必要に応じて退職金の一部または全部を分割して支給することができる。</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="8" customHeight="1"/>
-    <row r="101" ht="8" customHeight="1">
-      <c r="A101" s="28" t="inlineStr"/>
-      <c r="B101" s="12" t="n"/>
-      <c r="C101" s="12" t="n"/>
-      <c r="D101" s="12" t="n"/>
-      <c r="E101" s="12" t="n"/>
-    </row>
-    <row r="102" ht="10" customHeight="1"/>
-    <row r="103" ht="30" customHeight="1">
-      <c r="A103" s="25" t="inlineStr">
-        <is>
-          <t>附則</t>
         </is>
       </c>
     </row>
     <row r="104" ht="20" customHeight="1">
       <c r="A104" s="27" t="inlineStr">
         <is>
+          <t>3　虚偽の申告により雇用契約を締結したことが判明した場合</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="8" customHeight="1"/>
+    <row r="106" ht="20" customHeight="1">
+      <c r="A106" s="26" t="inlineStr">
+        <is>
+          <t>（支給手続）</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="20" customHeight="1">
+      <c r="A107" s="27" t="inlineStr">
+        <is>
+          <t>第16条　退職金は、退職日から2か月以内に本人の指定口座に振り込む。</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="20" customHeight="1">
+      <c r="A108" s="27" t="inlineStr">
+        <is>
+          <t>2　会社は、本人の同意を得た場合に限り、退職金を分割して支給することができる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="8" customHeight="1"/>
+    <row r="110" ht="8" customHeight="1">
+      <c r="A110" s="28" t="inlineStr"/>
+      <c r="B110" s="12" t="n"/>
+      <c r="C110" s="12" t="n"/>
+      <c r="D110" s="12" t="n"/>
+      <c r="E110" s="12" t="n"/>
+    </row>
+    <row r="111" ht="10" customHeight="1"/>
+    <row r="112" ht="30" customHeight="1">
+      <c r="A112" s="25" t="inlineStr">
+        <is>
+          <t>附則</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="20" customHeight="1">
+      <c r="A113" s="27" t="inlineStr">
+        <is>
           <t>1　本規程に定めのない事項は、就業規則その他関係規程による。</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="20" customHeight="1">
-      <c r="A105" s="27" t="inlineStr">
+    <row r="114" ht="20" customHeight="1">
+      <c r="A114" s="27" t="inlineStr">
         <is>
           <t>2　本規程は令和8年2月1日から施行する。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="57">
+  <mergeCells count="64">
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A34:E34"/>
     <mergeCell ref="A77:E77"/>
     <mergeCell ref="A59:E59"/>
     <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A73:E73"/>
+    <mergeCell ref="A83:E83"/>
+    <mergeCell ref="A114:E114"/>
     <mergeCell ref="A82:E82"/>
     <mergeCell ref="A60:E60"/>
-    <mergeCell ref="A98:E98"/>
+    <mergeCell ref="A49:E49"/>
     <mergeCell ref="A51:E51"/>
+    <mergeCell ref="A107:E107"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A45:E45"/>
-    <mergeCell ref="A94:E94"/>
     <mergeCell ref="A103:E103"/>
-    <mergeCell ref="A79:E79"/>
+    <mergeCell ref="A88:E88"/>
+    <mergeCell ref="A110:E110"/>
     <mergeCell ref="A69:E69"/>
+    <mergeCell ref="A87:E87"/>
     <mergeCell ref="A65:E65"/>
     <mergeCell ref="A78:E78"/>
-    <mergeCell ref="A54:E54"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A99:E99"/>
+    <mergeCell ref="A90:E90"/>
+    <mergeCell ref="A108:E108"/>
     <mergeCell ref="A37:E37"/>
-    <mergeCell ref="A75:E75"/>
+    <mergeCell ref="A84:E84"/>
+    <mergeCell ref="A66:E66"/>
     <mergeCell ref="A74:E74"/>
+    <mergeCell ref="A80:E80"/>
     <mergeCell ref="A56:E56"/>
     <mergeCell ref="A27:E27"/>
-    <mergeCell ref="A105:E105"/>
-    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="A55:E55"/>
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A57:E57"/>
-    <mergeCell ref="A95:E95"/>
     <mergeCell ref="A101:E101"/>
+    <mergeCell ref="A86:E86"/>
     <mergeCell ref="A104:E104"/>
+    <mergeCell ref="A113:E113"/>
     <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A76:E76"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="A71:E71"/>
     <mergeCell ref="A47:E47"/>
-    <mergeCell ref="A97:E97"/>
+    <mergeCell ref="A106:E106"/>
     <mergeCell ref="A53:E53"/>
     <mergeCell ref="A91:E91"/>
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A62:E62"/>
     <mergeCell ref="A43:E43"/>
     <mergeCell ref="A81:E81"/>
+    <mergeCell ref="A100:E100"/>
     <mergeCell ref="A72:E72"/>
+    <mergeCell ref="A52:E52"/>
     <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A112:E112"/>
     <mergeCell ref="A68:E68"/>
     <mergeCell ref="A63:E63"/>
-    <mergeCell ref="A93:E93"/>
+    <mergeCell ref="A102:E102"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A31:E31"/>
     <mergeCell ref="A44:E44"/>
     <mergeCell ref="A40:E40"/>
-    <mergeCell ref="A67:E67"/>
-    <mergeCell ref="A92:E92"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6683,7 +6926,7 @@
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>4 サービス利用料金は１か月ごとに計算し、事業者が届ける請求書により、利用者は下記の方法により翌月26日までに支払うものとし、支払いを受けたときは領収証を発行します。</t>
+          <t>4 サービス利用料金は１か月ごとに計算し、事業者が届ける請求書により、利用者は下記の方法により重要事項説明書に定める期日までに支払うものとし、支払いを受けたときは領収証を発行します。</t>
         </is>
       </c>
     </row>
@@ -7019,7 +7262,7 @@
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="9" t="inlineStr">
         <is>
-          <t>一 利用者がこの契約に定める利用料等の支払いを３か月以上遅延し、文書による支払い催告を行ったにもかかわらず、催告の日から７日以内にその支払いがなかった場合</t>
+          <t>一 利用者がこの契約に定める利用料等の支払いを３か月以上遅延し、文書による支払い催告を行ったにもかかわらず、催告の日から30日以内にその支払いがなかった場合</t>
         </is>
       </c>
     </row>
@@ -7393,7 +7636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7434,7 +7677,7 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t>（1）障害福祉/高齢者介護サービスの提供のため</t>
+          <t>（1）介護サービスの提供のため</t>
         </is>
       </c>
     </row>
@@ -7476,7 +7719,7 @@
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>事業所は、障害福祉サービスを円滑に提供するため下記の事業者、機関等へ個人情報を提供することがあります。</t>
+          <t>事業所は、介護サービスを円滑に提供するため下記の事業者、機関等へ個人情報を提供することがあります。</t>
         </is>
       </c>
     </row>
@@ -7508,133 +7751,125 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1">
+    <row r="21" ht="32" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>居宅介護・重度訪問介護契約書の第２条に定める契約期間及び法令の定めるところによる当該</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>契約の解約又は解除後の書類保存期間に相当する期間使用します。</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
+          <t>指定訪問介護契約書の第２条に定める契約期間、及び法令の定めるところによる当該契約の解約又は解除後の書類保存期間に相当する期間使用します。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>日付</t>
         </is>
       </c>
-      <c r="B26" s="18" t="inlineStr">
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">　　　　年　　月　　日</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="19" t="inlineStr">
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="19" t="inlineStr">
         <is>
           <t>利用者</t>
         </is>
       </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="B27" s="20" t="inlineStr">
+        <is>
+          <t>（住所）</t>
+        </is>
+      </c>
+      <c r="C27" s="21" t="inlineStr"/>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="12" t="n"/>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="B28" s="20" t="inlineStr"/>
+      <c r="C28" s="21" t="inlineStr"/>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="12" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="B29" s="20" t="inlineStr">
         <is>
-          <t>（住所）</t>
-        </is>
-      </c>
-      <c r="C29" s="21" t="inlineStr"/>
+          <t>（氏名）</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　　　　　　　　　　　　　　印</t>
+        </is>
+      </c>
       <c r="D29" s="12" t="n"/>
       <c r="E29" s="12" t="n"/>
     </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="B30" s="20" t="inlineStr"/>
-      <c r="C30" s="21" t="inlineStr"/>
-      <c r="D30" s="12" t="n"/>
-      <c r="E30" s="12" t="n"/>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="B31" s="20" t="inlineStr">
-        <is>
-          <t>（氏名）</t>
-        </is>
-      </c>
-      <c r="C31" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　　　　　　　　　　　　　　印</t>
-        </is>
-      </c>
-      <c r="D31" s="12" t="n"/>
-      <c r="E31" s="12" t="n"/>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="19" t="inlineStr">
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="19" t="inlineStr">
         <is>
           <t>（代理人または立会人等）</t>
         </is>
       </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>（住所）</t>
+        </is>
+      </c>
+      <c r="C32" s="21" t="inlineStr"/>
+      <c r="D32" s="12" t="n"/>
+      <c r="E32" s="12" t="n"/>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="B33" s="20" t="inlineStr"/>
+      <c r="C33" s="21" t="inlineStr"/>
+      <c r="D33" s="12" t="n"/>
+      <c r="E33" s="12" t="n"/>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="B34" s="20" t="inlineStr">
         <is>
-          <t>（住所）</t>
-        </is>
-      </c>
-      <c r="C34" s="21" t="inlineStr"/>
+          <t>（氏名）</t>
+        </is>
+      </c>
+      <c r="C34" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　　　　　　　　　　　　　　印</t>
+        </is>
+      </c>
       <c r="D34" s="12" t="n"/>
       <c r="E34" s="12" t="n"/>
     </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="B35" s="20" t="inlineStr"/>
-      <c r="C35" s="21" t="inlineStr"/>
-      <c r="D35" s="12" t="n"/>
-      <c r="E35" s="12" t="n"/>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="B36" s="20" t="inlineStr">
-        <is>
-          <t>（氏名）</t>
-        </is>
-      </c>
-      <c r="C36" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　　　　　　　　　　　　　　印</t>
-        </is>
-      </c>
-      <c r="D36" s="12" t="n"/>
-      <c r="E36" s="12" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="26">
-    <mergeCell ref="C29:E29"/>
+  <mergeCells count="25">
     <mergeCell ref="A15:E15"/>
-    <mergeCell ref="C31:E31"/>
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="C27:E27"/>
     <mergeCell ref="A16:E16"/>
     <mergeCell ref="A7:E7"/>
     <mergeCell ref="A18:E18"/>
+    <mergeCell ref="C32:E32"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A21:E21"/>
     <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="A26:E26"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A23:E23"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="A8:E8"/>
-    <mergeCell ref="C30:E30"/>
     <mergeCell ref="C34:E34"/>
     <mergeCell ref="A17:E17"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="C33:E33"/>
     <mergeCell ref="A20:E20"/>
     <mergeCell ref="A10:E10"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="A31:E31"/>
     <mergeCell ref="A9:E9"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
@@ -8937,7 +9172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E113"/>
+  <dimension ref="A1:E114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -9074,456 +9309,464 @@
     <row r="41" ht="32" customHeight="1">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>第4条　会社は、常時50人未満の事業場であるため法令上の衛生管理者選任義務はないが、必要に応じて衛生推進者を指名し、従業員の健康保持増進活動を推進することができる。</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="8" customHeight="1"/>
-    <row r="43" ht="8" customHeight="1">
-      <c r="A43" s="28" t="inlineStr"/>
-      <c r="B43" s="12" t="n"/>
-      <c r="C43" s="12" t="n"/>
-      <c r="D43" s="12" t="n"/>
-      <c r="E43" s="12" t="n"/>
-    </row>
-    <row r="44" ht="10" customHeight="1"/>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="25" t="inlineStr">
+          <t>第4条　会社は、常時10人以上50人未満の労働者を使用する事業場として、労働安全衛生法に基づき衛生推進者を選任し、その氏名を事業場に掲示して従業員に周知する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="27" t="inlineStr">
+        <is>
+          <t>2　衛生推進者は、健康診断、職場環境の点検、安全衛生教育その他衛生に関する業務を担当する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="8" customHeight="1"/>
+    <row r="44" ht="8" customHeight="1">
+      <c r="A44" s="28" t="inlineStr"/>
+      <c r="B44" s="12" t="n"/>
+      <c r="C44" s="12" t="n"/>
+      <c r="D44" s="12" t="n"/>
+      <c r="E44" s="12" t="n"/>
+    </row>
+    <row r="45" ht="10" customHeight="1"/>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="25" t="inlineStr">
         <is>
           <t>第3章　健康管理</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="26" t="inlineStr">
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="26" t="inlineStr">
         <is>
           <t>（健康診断）</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="27" t="inlineStr">
-        <is>
-          <t>第5条　会社は、労働安全衛生法に基づき、従業員に次の健康診断を実施する。</t>
         </is>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>1　雇入時健康診断（入社時）</t>
+          <t>第5条　会社は、労働安全衛生法に基づき、従業員に次の健康診断を実施する。</t>
         </is>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>2　定期健康診断（年1回。ただし夜勤業務に従事する者については年2回）</t>
+          <t>1　雇入時健康診断（入社時）</t>
         </is>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>3　特定業務従事者健康診断（必要に応じて）</t>
+          <t>2　定期健康診断（年1回。ただし夜勤業務に従事する者については年2回）</t>
         </is>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="27" t="inlineStr">
         <is>
+          <t>3　特定業務従事者健康診断（必要に応じて）</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="27" t="inlineStr">
+        <is>
           <t>2　健康診断の費用は会社が負担する。</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="8" customHeight="1"/>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="26" t="inlineStr">
+    <row r="53" ht="8" customHeight="1"/>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="26" t="inlineStr">
         <is>
           <t>（診断結果への対応）</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="32" customHeight="1">
-      <c r="A54" s="27" t="inlineStr">
+    <row r="55" ht="32" customHeight="1">
+      <c r="A55" s="27" t="inlineStr">
         <is>
           <t>第6条　会社は、健康診断の結果に基づき、必要に応じて就業上の措置を講じる。従業員は医師の意見に従い、就業制限や治療を受けなければならない。</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="8" customHeight="1"/>
-    <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="26" t="inlineStr">
+    <row r="56" ht="8" customHeight="1"/>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="26" t="inlineStr">
         <is>
           <t>（ストレスチェック）</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="32" customHeight="1">
-      <c r="A57" s="27" t="inlineStr">
+    <row r="58" ht="32" customHeight="1">
+      <c r="A58" s="27" t="inlineStr">
         <is>
           <t>第7条　会社は、従業員数50人未満のため法定義務はないが、必要に応じてストレスチェックを実施し、結果に基づき職場環境改善や個別対応を行うことができる。</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="8" customHeight="1"/>
-    <row r="59" ht="8" customHeight="1">
-      <c r="A59" s="28" t="inlineStr"/>
-      <c r="B59" s="12" t="n"/>
-      <c r="C59" s="12" t="n"/>
-      <c r="D59" s="12" t="n"/>
-      <c r="E59" s="12" t="n"/>
-    </row>
-    <row r="60" ht="10" customHeight="1"/>
-    <row r="61" ht="30" customHeight="1">
-      <c r="A61" s="25" t="inlineStr">
+    <row r="59" ht="8" customHeight="1"/>
+    <row r="60" ht="8" customHeight="1">
+      <c r="A60" s="28" t="inlineStr"/>
+      <c r="B60" s="12" t="n"/>
+      <c r="C60" s="12" t="n"/>
+      <c r="D60" s="12" t="n"/>
+      <c r="E60" s="12" t="n"/>
+    </row>
+    <row r="61" ht="10" customHeight="1"/>
+    <row r="62" ht="30" customHeight="1">
+      <c r="A62" s="25" t="inlineStr">
         <is>
           <t>第4章　職場環境の整備</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="20" customHeight="1">
-      <c r="A62" s="26" t="inlineStr">
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="26" t="inlineStr">
         <is>
           <t>（作業環境管理）</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="27" t="inlineStr">
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="27" t="inlineStr">
         <is>
           <t>第8条　会社は、職場の換気、採光、照明、温度、騒音等の環境を適正に維持する。</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="8" customHeight="1"/>
-    <row r="65" ht="20" customHeight="1">
-      <c r="A65" s="26" t="inlineStr">
+    <row r="65" ht="8" customHeight="1"/>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="26" t="inlineStr">
         <is>
           <t>（作業方法の改善）</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="32" customHeight="1">
-      <c r="A66" s="27" t="inlineStr">
-        <is>
-          <t>第9条　会社は、業務に伴う危険や健康障害を防止するため、作業方法を改善し、安全衛生教育を実施する。</t>
         </is>
       </c>
     </row>
     <row r="67" ht="32" customHeight="1">
       <c r="A67" s="27" t="inlineStr">
         <is>
+          <t>第9条　会社は、業務に伴う危険や健康障害を防止するため、作業方法を改善し、安全衛生教育を実施する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="32" customHeight="1">
+      <c r="A68" s="27" t="inlineStr">
+        <is>
           <t>2　特に介護業務においては、腰痛予防、福祉用具の適切な使用、送迎業務における車両運転の安全確保に努める。</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="8" customHeight="1"/>
-    <row r="69" ht="20" customHeight="1">
-      <c r="A69" s="26" t="inlineStr">
+    <row r="69" ht="8" customHeight="1"/>
+    <row r="70" ht="20" customHeight="1">
+      <c r="A70" s="26" t="inlineStr">
         <is>
           <t>（感染症予防）</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="32" customHeight="1">
-      <c r="A70" s="27" t="inlineStr">
+    <row r="71" ht="32" customHeight="1">
+      <c r="A71" s="27" t="inlineStr">
         <is>
           <t>第10条　会社は、インフルエンザ、新型コロナウイルスその他感染症の予防に努め、必要に応じてマスク着用、手指消毒、在宅勤務、出勤停止等の措置を講じる。</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="8" customHeight="1"/>
-    <row r="72" ht="8" customHeight="1">
-      <c r="A72" s="28" t="inlineStr"/>
-      <c r="B72" s="12" t="n"/>
-      <c r="C72" s="12" t="n"/>
-      <c r="D72" s="12" t="n"/>
-      <c r="E72" s="12" t="n"/>
-    </row>
-    <row r="73" ht="10" customHeight="1"/>
-    <row r="74" ht="30" customHeight="1">
-      <c r="A74" s="25" t="inlineStr">
+    <row r="72" ht="8" customHeight="1"/>
+    <row r="73" ht="8" customHeight="1">
+      <c r="A73" s="28" t="inlineStr"/>
+      <c r="B73" s="12" t="n"/>
+      <c r="C73" s="12" t="n"/>
+      <c r="D73" s="12" t="n"/>
+      <c r="E73" s="12" t="n"/>
+    </row>
+    <row r="74" ht="10" customHeight="1"/>
+    <row r="75" ht="30" customHeight="1">
+      <c r="A75" s="25" t="inlineStr">
         <is>
           <t>第5章　安全衛生教育</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="26" t="inlineStr">
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="26" t="inlineStr">
         <is>
           <t>（教育の実施）</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="20" customHeight="1">
-      <c r="A76" s="27" t="inlineStr">
-        <is>
-          <t>第11条　会社は、従業員に対して次の安全衛生教育を実施する。</t>
         </is>
       </c>
     </row>
     <row r="77" ht="20" customHeight="1">
       <c r="A77" s="27" t="inlineStr">
         <is>
-          <t>1　雇入時教育（安全衛生に関する基本事項）</t>
+          <t>第11条　会社は、従業員に対して次の安全衛生教育を実施する。</t>
         </is>
       </c>
     </row>
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="27" t="inlineStr">
         <is>
-          <t>2　配置転換時教育（新しい業務に伴う危険防止）</t>
+          <t>1　雇入時教育（安全衛生に関する基本事項）</t>
         </is>
       </c>
     </row>
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="27" t="inlineStr">
         <is>
-          <t>3　作業内容変更時教育（介護・送迎業務における腰痛防止、交通安全等）</t>
+          <t>2　配置転換時教育（新しい業務に伴う危険防止）</t>
         </is>
       </c>
     </row>
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="27" t="inlineStr">
         <is>
+          <t>3　作業内容変更時教育（介護・送迎業務における腰痛防止、交通安全等）</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="20" customHeight="1">
+      <c r="A81" s="27" t="inlineStr">
+        <is>
           <t>4　定期教育（年1回以上、安全衛生全般に関する教育）</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="8" customHeight="1"/>
-    <row r="82" ht="8" customHeight="1">
-      <c r="A82" s="28" t="inlineStr"/>
-      <c r="B82" s="12" t="n"/>
-      <c r="C82" s="12" t="n"/>
-      <c r="D82" s="12" t="n"/>
-      <c r="E82" s="12" t="n"/>
-    </row>
-    <row r="83" ht="10" customHeight="1"/>
-    <row r="84" ht="30" customHeight="1">
-      <c r="A84" s="25" t="inlineStr">
+    <row r="82" ht="8" customHeight="1"/>
+    <row r="83" ht="8" customHeight="1">
+      <c r="A83" s="28" t="inlineStr"/>
+      <c r="B83" s="12" t="n"/>
+      <c r="C83" s="12" t="n"/>
+      <c r="D83" s="12" t="n"/>
+      <c r="E83" s="12" t="n"/>
+    </row>
+    <row r="84" ht="10" customHeight="1"/>
+    <row r="85" ht="30" customHeight="1">
+      <c r="A85" s="25" t="inlineStr">
         <is>
           <t>第6章　労働災害への対応</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="20" customHeight="1">
-      <c r="A85" s="26" t="inlineStr">
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="26" t="inlineStr">
         <is>
           <t>（災害発生時の措置）</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="32" customHeight="1">
-      <c r="A86" s="27" t="inlineStr">
+    <row r="87" ht="32" customHeight="1">
+      <c r="A87" s="27" t="inlineStr">
         <is>
           <t>第12条　労働災害が発生した場合、従業員は直ちに上長に報告し、会社は応急措置を講じ、必要に応じて関係行政官庁へ報告する。</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="8" customHeight="1"/>
-    <row r="88" ht="20" customHeight="1">
-      <c r="A88" s="26" t="inlineStr">
+    <row r="88" ht="8" customHeight="1"/>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="26" t="inlineStr">
         <is>
           <t>（再発防止）</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="20" customHeight="1">
-      <c r="A89" s="27" t="inlineStr">
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="27" t="inlineStr">
         <is>
           <t>第13条　会社は、労働災害が発生した場合、その原因を調査し、再発防止策を講じる。</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="8" customHeight="1"/>
-    <row r="91" ht="8" customHeight="1">
-      <c r="A91" s="28" t="inlineStr"/>
-      <c r="B91" s="12" t="n"/>
-      <c r="C91" s="12" t="n"/>
-      <c r="D91" s="12" t="n"/>
-      <c r="E91" s="12" t="n"/>
-    </row>
-    <row r="92" ht="10" customHeight="1"/>
-    <row r="93" ht="30" customHeight="1">
-      <c r="A93" s="25" t="inlineStr">
+    <row r="91" ht="8" customHeight="1"/>
+    <row r="92" ht="8" customHeight="1">
+      <c r="A92" s="28" t="inlineStr"/>
+      <c r="B92" s="12" t="n"/>
+      <c r="C92" s="12" t="n"/>
+      <c r="D92" s="12" t="n"/>
+      <c r="E92" s="12" t="n"/>
+    </row>
+    <row r="93" ht="10" customHeight="1"/>
+    <row r="94" ht="30" customHeight="1">
+      <c r="A94" s="25" t="inlineStr">
         <is>
           <t>第7章　健康保持・メンタルヘルス</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="20" customHeight="1">
-      <c r="A94" s="26" t="inlineStr">
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="26" t="inlineStr">
         <is>
           <t>（過重労働対策）</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="32" customHeight="1">
-      <c r="A95" s="27" t="inlineStr">
+    <row r="96" ht="32" customHeight="1">
+      <c r="A96" s="27" t="inlineStr">
         <is>
           <t>第14条　会社は、時間外労働や深夜労働が従業員の心身に過度の負担を与えないように管理し、長時間労働が認められる場合は速やかに対応する。</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="8" customHeight="1"/>
-    <row r="97" ht="20" customHeight="1">
-      <c r="A97" s="26" t="inlineStr">
+    <row r="97" ht="8" customHeight="1"/>
+    <row r="98" ht="20" customHeight="1">
+      <c r="A98" s="26" t="inlineStr">
         <is>
           <t>（メンタルヘルス対応）</t>
         </is>
       </c>
     </row>
-    <row r="98" ht="32" customHeight="1">
-      <c r="A98" s="27" t="inlineStr">
+    <row r="99" ht="32" customHeight="1">
+      <c r="A99" s="27" t="inlineStr">
         <is>
           <t>第15条　会社は、従業員がうつ病、適応障害その他のメンタル不調を抱えた場合、医師の診断や専門家の意見を踏まえ、必要な就業上の措置（休職・勤務軽減・復職支援等）を講じる。</t>
         </is>
       </c>
     </row>
-    <row r="99" ht="8" customHeight="1"/>
-    <row r="100" ht="8" customHeight="1">
-      <c r="A100" s="28" t="inlineStr"/>
-      <c r="B100" s="12" t="n"/>
-      <c r="C100" s="12" t="n"/>
-      <c r="D100" s="12" t="n"/>
-      <c r="E100" s="12" t="n"/>
-    </row>
-    <row r="101" ht="10" customHeight="1"/>
-    <row r="102" ht="30" customHeight="1">
-      <c r="A102" s="25" t="inlineStr">
+    <row r="100" ht="8" customHeight="1"/>
+    <row r="101" ht="8" customHeight="1">
+      <c r="A101" s="28" t="inlineStr"/>
+      <c r="B101" s="12" t="n"/>
+      <c r="C101" s="12" t="n"/>
+      <c r="D101" s="12" t="n"/>
+      <c r="E101" s="12" t="n"/>
+    </row>
+    <row r="102" ht="10" customHeight="1"/>
+    <row r="103" ht="30" customHeight="1">
+      <c r="A103" s="25" t="inlineStr">
         <is>
           <t>第8章　その他</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="20" customHeight="1">
-      <c r="A103" s="26" t="inlineStr">
+    <row r="104" ht="20" customHeight="1">
+      <c r="A104" s="26" t="inlineStr">
         <is>
           <t>（健康情報の管理）</t>
         </is>
       </c>
     </row>
-    <row r="104" ht="32" customHeight="1">
-      <c r="A104" s="27" t="inlineStr">
+    <row r="105" ht="32" customHeight="1">
+      <c r="A105" s="27" t="inlineStr">
         <is>
           <t>第16条　健康診断やストレスチェックの結果、相談等により得た従業員の個人情報は厳格に管理し、本人の同意なく第三者に開示してはならない。</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="8" customHeight="1"/>
-    <row r="106" ht="20" customHeight="1">
-      <c r="A106" s="26" t="inlineStr">
+    <row r="106" ht="8" customHeight="1"/>
+    <row r="107" ht="20" customHeight="1">
+      <c r="A107" s="26" t="inlineStr">
         <is>
           <t>（不利益取扱いの禁止）</t>
         </is>
       </c>
     </row>
-    <row r="107" ht="32" customHeight="1">
-      <c r="A107" s="27" t="inlineStr">
+    <row r="108" ht="32" customHeight="1">
+      <c r="A108" s="27" t="inlineStr">
         <is>
           <t>第17条　会社は、従業員が健康診断、感染症予防措置、安全衛生教育等を受けたことを理由に、不利益取扱いをしてはならない。</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="8" customHeight="1"/>
-    <row r="109" ht="8" customHeight="1">
-      <c r="A109" s="28" t="inlineStr"/>
-      <c r="B109" s="12" t="n"/>
-      <c r="C109" s="12" t="n"/>
-      <c r="D109" s="12" t="n"/>
-      <c r="E109" s="12" t="n"/>
-    </row>
-    <row r="110" ht="10" customHeight="1"/>
-    <row r="111" ht="30" customHeight="1">
-      <c r="A111" s="25" t="inlineStr">
+    <row r="109" ht="8" customHeight="1"/>
+    <row r="110" ht="8" customHeight="1">
+      <c r="A110" s="28" t="inlineStr"/>
+      <c r="B110" s="12" t="n"/>
+      <c r="C110" s="12" t="n"/>
+      <c r="D110" s="12" t="n"/>
+      <c r="E110" s="12" t="n"/>
+    </row>
+    <row r="111" ht="10" customHeight="1"/>
+    <row r="112" ht="30" customHeight="1">
+      <c r="A112" s="25" t="inlineStr">
         <is>
           <t>附則</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="20" customHeight="1">
-      <c r="A112" s="27" t="inlineStr">
-        <is>
-          <t>1　本規程に定めのない事項は、労働基準法、労働安全衛生法その他関係法令による。</t>
         </is>
       </c>
     </row>
     <row r="113" ht="20" customHeight="1">
       <c r="A113" s="27" t="inlineStr">
         <is>
+          <t>1　本規程に定めのない事項は、労働基準法、労働安全衛生法その他関係法令による。</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="20" customHeight="1">
+      <c r="A114" s="27" t="inlineStr">
+        <is>
           <t>2　本規程は令和8年2月1日から施行する。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="66">
+  <mergeCells count="67">
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A77:E77"/>
-    <mergeCell ref="A59:E59"/>
+    <mergeCell ref="A83:E83"/>
+    <mergeCell ref="A114:E114"/>
     <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A82:E82"/>
+    <mergeCell ref="A73:E73"/>
+    <mergeCell ref="A64:E64"/>
+    <mergeCell ref="A60:E60"/>
     <mergeCell ref="A98:E98"/>
     <mergeCell ref="A49:E49"/>
     <mergeCell ref="A51:E51"/>
     <mergeCell ref="A107:E107"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A45:E45"/>
     <mergeCell ref="A94:E94"/>
+    <mergeCell ref="A103:E103"/>
     <mergeCell ref="A36:E36"/>
-    <mergeCell ref="A103:E103"/>
-    <mergeCell ref="A61:E61"/>
-    <mergeCell ref="A88:E88"/>
     <mergeCell ref="A70:E70"/>
     <mergeCell ref="A79:E79"/>
-    <mergeCell ref="A69:E69"/>
-    <mergeCell ref="A65:E65"/>
+    <mergeCell ref="A110:E110"/>
+    <mergeCell ref="A87:E87"/>
     <mergeCell ref="A78:E78"/>
     <mergeCell ref="A54:E54"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A90:E90"/>
+    <mergeCell ref="A108:E108"/>
+    <mergeCell ref="A99:E99"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="A46:E46"/>
     <mergeCell ref="A75:E75"/>
     <mergeCell ref="A66:E66"/>
-    <mergeCell ref="A84:E84"/>
     <mergeCell ref="A89:E89"/>
-    <mergeCell ref="A74:E74"/>
     <mergeCell ref="A80:E80"/>
-    <mergeCell ref="A56:E56"/>
     <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A105:E105"/>
+    <mergeCell ref="A55:E55"/>
     <mergeCell ref="A50:E50"/>
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A57:E57"/>
     <mergeCell ref="A95:E95"/>
     <mergeCell ref="A86:E86"/>
+    <mergeCell ref="A101:E101"/>
     <mergeCell ref="A104:E104"/>
+    <mergeCell ref="A42:E42"/>
     <mergeCell ref="A113:E113"/>
     <mergeCell ref="A76:E76"/>
     <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A71:E71"/>
     <mergeCell ref="A47:E47"/>
     <mergeCell ref="A85:E85"/>
-    <mergeCell ref="A97:E97"/>
-    <mergeCell ref="A106:E106"/>
-    <mergeCell ref="A53:E53"/>
-    <mergeCell ref="A91:E91"/>
     <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A109:E109"/>
     <mergeCell ref="A62:E62"/>
-    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A81:E81"/>
     <mergeCell ref="A38:E38"/>
-    <mergeCell ref="A100:E100"/>
-    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="A96:E96"/>
+    <mergeCell ref="A52:E52"/>
     <mergeCell ref="A28:E28"/>
     <mergeCell ref="A112:E112"/>
+    <mergeCell ref="A68:E68"/>
     <mergeCell ref="A63:E63"/>
-    <mergeCell ref="A102:E102"/>
-    <mergeCell ref="A93:E93"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A31:E31"/>
-    <mergeCell ref="A111:E111"/>
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A58:E58"/>
     <mergeCell ref="A40:E40"/>
     <mergeCell ref="A67:E67"/>
+    <mergeCell ref="A92:E92"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9907,7 +10150,7 @@
     <row r="77" ht="20" customHeight="1">
       <c r="A77" s="27" t="inlineStr">
         <is>
-          <t>3　禁錮以上の刑に処せられ、その判決が確定した場合。</t>
+          <t>3　拘禁刑以上の刑に処せられ、その判決が確定した場合。</t>
         </is>
       </c>
     </row>
@@ -10675,7 +10918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E133"/>
+  <dimension ref="A1:E146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -10794,267 +11037,273 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="20" customHeight="1">
+    <row r="38" ht="32" customHeight="1">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>2　その後も、継続勤務ごとに6か月経過するごとに10日の年次有給休暇を付与する。</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="8" customHeight="1"/>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="26" t="inlineStr">
+          <t>2　その後は、継続勤務年数に応じ、1年ごとに次の日数を付与する。ただし、直前の1年間の全労働日の8割以上出勤した者に限る。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="32" customHeight="1">
+      <c r="A39" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　継続勤務1年6か月：11日　2年6か月：12日　3年6か月：14日　4年6か月：16日　5年6か月：18日　6年6か月以上：20日</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="32" customHeight="1">
+      <c r="A40" s="27" t="inlineStr">
+        <is>
+          <t>3　週所定労働日数が4日以下かつ週所定労働時間が30時間未満の従業員には、労働基準法第39条第3項に定める日数を比例付与する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="8" customHeight="1"/>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="26" t="inlineStr">
         <is>
           <t>（取得方法）</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="32" customHeight="1">
-      <c r="A41" s="27" t="inlineStr">
+    <row r="43" ht="32" customHeight="1">
+      <c r="A43" s="27" t="inlineStr">
         <is>
           <t>第4条　年次有給休暇の取得は、従業員の請求による。会社は業務の正常な運営を妨げる場合を除き、これを認めなければならない。</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="8" customHeight="1"/>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="26" t="inlineStr">
+    <row r="44" ht="8" customHeight="1"/>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="26" t="inlineStr">
         <is>
           <t>（時季変更権）</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="27" t="inlineStr">
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="27" t="inlineStr">
         <is>
           <t>第5条　会社は、業務の正常な運営を妨げる場合、休暇の取得時季を変更することができる。</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="8" customHeight="1"/>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="26" t="inlineStr">
+    <row r="47" ht="8" customHeight="1"/>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="26" t="inlineStr">
         <is>
           <t>（時間単位年休）</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="32" customHeight="1">
-      <c r="A47" s="27" t="inlineStr">
-        <is>
-          <t>第6条　会社は、労使協定を締結した場合に限り、年次有給休暇の一部を時間単位で取得させることができる。</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="8" customHeight="1"/>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="26" t="inlineStr">
+    <row r="49" ht="32" customHeight="1">
+      <c r="A49" s="27" t="inlineStr">
+        <is>
+          <t>第6条　会社は、労使協定を締結した場合に限り、年次有給休暇のうち年5日の範囲内で、時間単位で取得させることができる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="8" customHeight="1"/>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="26" t="inlineStr">
         <is>
           <t>（計画的付与）</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="27" t="inlineStr">
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="27" t="inlineStr">
         <is>
           <t>第7条　会社は、労使協定に基づき、年次有給休暇の一部を計画的に付与することができる。</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="8" customHeight="1"/>
-    <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="26" t="inlineStr">
+    <row r="53" ht="8" customHeight="1"/>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="26" t="inlineStr">
         <is>
           <t>（年5日の取得義務）</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="32" customHeight="1">
-      <c r="A53" s="27" t="inlineStr">
+    <row r="55" ht="32" customHeight="1">
+      <c r="A55" s="27" t="inlineStr">
         <is>
           <t>第8条　会社は、年次有給休暇のうち年間5日については、従業員が必ず取得するよう管理しなければならない。</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="27" t="inlineStr">
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="27" t="inlineStr">
         <is>
           <t>2　従業員が自ら請求しない場合、会社は取得時季を指定して取得させる。</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="8" customHeight="1"/>
-    <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="26" t="inlineStr">
+    <row r="57" ht="8" customHeight="1"/>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="26" t="inlineStr">
         <is>
           <t>（有効期限）</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="27" t="inlineStr">
-        <is>
-          <t>第9条　年次有給休暇の有効期限は、付与日から2年間とする。</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="27" t="inlineStr">
-        <is>
-          <t>2　繰越は1年間に限り認められるが、2年を経過した分については消滅する。</t>
         </is>
       </c>
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="27" t="inlineStr">
         <is>
+          <t>第9条　年次有給休暇の有効期限は、付与日から2年間とする。</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="27" t="inlineStr">
+        <is>
+          <t>2　繰越は1年間に限り認められるが、2年を経過した分については消滅する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="27" t="inlineStr">
+        <is>
           <t>3　消滅した年次有給休暇については、会社は金銭その他の補償を行わない。</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="8" customHeight="1"/>
-    <row r="61" ht="8" customHeight="1">
-      <c r="A61" s="28" t="inlineStr"/>
-      <c r="B61" s="12" t="n"/>
-      <c r="C61" s="12" t="n"/>
-      <c r="D61" s="12" t="n"/>
-      <c r="E61" s="12" t="n"/>
-    </row>
-    <row r="62" ht="10" customHeight="1"/>
-    <row r="63" ht="30" customHeight="1">
-      <c r="A63" s="25" t="inlineStr">
+    <row r="62" ht="8" customHeight="1"/>
+    <row r="63" ht="8" customHeight="1">
+      <c r="A63" s="28" t="inlineStr"/>
+      <c r="B63" s="12" t="n"/>
+      <c r="C63" s="12" t="n"/>
+      <c r="D63" s="12" t="n"/>
+      <c r="E63" s="12" t="n"/>
+    </row>
+    <row r="64" ht="10" customHeight="1"/>
+    <row r="65" ht="30" customHeight="1">
+      <c r="A65" s="25" t="inlineStr">
         <is>
           <t>第3章　特別休暇</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="26" t="inlineStr">
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="26" t="inlineStr">
         <is>
           <t>（慶弔休暇）</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="20" customHeight="1">
-      <c r="A65" s="27" t="inlineStr">
-        <is>
-          <t>第10条　従業員に対し、次の慶弔休暇を付与する。</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="20" customHeight="1">
-      <c r="A66" s="27" t="inlineStr">
-        <is>
-          <t>1　本人の結婚：5日</t>
         </is>
       </c>
     </row>
     <row r="67" ht="20" customHeight="1">
       <c r="A67" s="27" t="inlineStr">
         <is>
-          <t>2　子女の結婚：2日</t>
+          <t>第10条　従業員に対し、次の慶弔休暇を付与する。</t>
         </is>
       </c>
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="27" t="inlineStr">
         <is>
-          <t>3　配偶者の死亡：5日</t>
+          <t>1　本人の結婚：5日</t>
         </is>
       </c>
     </row>
     <row r="69" ht="20" customHeight="1">
       <c r="A69" s="27" t="inlineStr">
         <is>
-          <t>4　父母・子の死亡：5日</t>
+          <t>2　子女の結婚：2日</t>
         </is>
       </c>
     </row>
     <row r="70" ht="20" customHeight="1">
       <c r="A70" s="27" t="inlineStr">
         <is>
-          <t>5　祖父母・兄弟姉妹の死亡：3日</t>
+          <t>3　配偶者の死亡：5日</t>
         </is>
       </c>
     </row>
     <row r="71" ht="20" customHeight="1">
       <c r="A71" s="27" t="inlineStr">
         <is>
-          <t>6　その他会社が必要と認めた場合：別途定める</t>
+          <t>4　父母・子の死亡：5日</t>
         </is>
       </c>
     </row>
     <row r="72" ht="20" customHeight="1">
       <c r="A72" s="27" t="inlineStr">
         <is>
+          <t>5　祖父母・兄弟姉妹の死亡：3日</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="27" t="inlineStr">
+        <is>
+          <t>6　その他会社が必要と認めた場合：別途定める</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="27" t="inlineStr">
+        <is>
           <t>2　慶弔休暇に伴う見舞金・祝い金等は「福利厚生規程」に定める。</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="8" customHeight="1"/>
-    <row r="74" ht="20" customHeight="1">
-      <c r="A74" s="26" t="inlineStr">
+    <row r="75" ht="8" customHeight="1"/>
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="26" t="inlineStr">
         <is>
           <t>（産前産後休業）</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="32" customHeight="1">
-      <c r="A75" s="27" t="inlineStr">
+    <row r="77" ht="32" customHeight="1">
+      <c r="A77" s="27" t="inlineStr">
         <is>
           <t>第11条　従業員が出産する場合は、労働基準法に基づき産前6週間（多胎妊娠の場合は14週間）、産後8週間を休業とする。</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="8" customHeight="1"/>
-    <row r="77" ht="20" customHeight="1">
-      <c r="A77" s="26" t="inlineStr">
+    <row r="78" ht="8" customHeight="1"/>
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="26" t="inlineStr">
         <is>
           <t>（育児休業・介護休業）</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="32" customHeight="1">
-      <c r="A78" s="27" t="inlineStr">
+    <row r="80" ht="32" customHeight="1">
+      <c r="A80" s="27" t="inlineStr">
         <is>
           <t>第12条　従業員は、育児・介護休業法に基づき、育児休業及び介護休業を取得することができる。期間・条件等は同法および「育児・介護休業規程」による。</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="8" customHeight="1"/>
-    <row r="80" ht="20" customHeight="1">
-      <c r="A80" s="26" t="inlineStr">
-        <is>
-          <t>（子の看護休暇・介護休暇）</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="32" customHeight="1">
-      <c r="A81" s="27" t="inlineStr">
-        <is>
-          <t>第13条　従業員は、小学校就学前の子1人につき年間5日（2人以上は10日）の子の看護休暇を取得できる。</t>
-        </is>
-      </c>
-    </row>
+    <row r="81" ht="8" customHeight="1"/>
     <row r="82" ht="20" customHeight="1">
-      <c r="A82" s="27" t="inlineStr">
-        <is>
-          <t>2　要介護家族については、年間5日の介護休暇を取得できる。</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="8" customHeight="1"/>
-    <row r="84" ht="20" customHeight="1">
-      <c r="A84" s="26" t="inlineStr">
-        <is>
-          <t>（病気休暇）</t>
+      <c r="A82" s="26" t="inlineStr">
+        <is>
+          <t>（子の看護等休暇・介護休暇）</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="32" customHeight="1">
+      <c r="A83" s="27" t="inlineStr">
+        <is>
+          <t>第13条　従業員は、小学校第3学年修了までの子を養育する場合、子1人につき年間5日（2人以上は10日）の子の看護等休暇を取得できる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="32" customHeight="1">
+      <c r="A84" s="27" t="inlineStr">
+        <is>
+          <t>2　要介護状態にある家族を介護する従業員は、対象家族1人につき年間5日（2人以上は10日）の介護休暇を取得できる。</t>
         </is>
       </c>
     </row>
     <row r="85" ht="32" customHeight="1">
       <c r="A85" s="27" t="inlineStr">
         <is>
-          <t>第14条　従業員が私傷病により就業できない場合は、会社の承認を得て病気休暇を与えることがある。日数や給与の取扱いは「休職規程」による。</t>
+          <t>3　子の看護等休暇及び介護休暇は、1日または時間単位で取得できる。詳細は「育児・介護休業規程」による。</t>
         </is>
       </c>
     </row>
@@ -11062,14 +11311,14 @@
     <row r="87" ht="20" customHeight="1">
       <c r="A87" s="26" t="inlineStr">
         <is>
-          <t>（公務・公用休暇）</t>
+          <t>（病気休暇）</t>
         </is>
       </c>
     </row>
     <row r="88" ht="32" customHeight="1">
       <c r="A88" s="27" t="inlineStr">
         <is>
-          <t>第15条　従業員が裁判員、証人、選挙、官公庁の要請による職務に従事する場合は、その期間を休暇とする。</t>
+          <t>第14条　従業員が私傷病により就業できない場合は、会社の承認を得て病気休暇を与えることがある。日数や給与の取扱いは「休職規程」による。</t>
         </is>
       </c>
     </row>
@@ -11077,14 +11326,14 @@
     <row r="90" ht="20" customHeight="1">
       <c r="A90" s="26" t="inlineStr">
         <is>
-          <t>（感染症予防に伴う休暇）</t>
+          <t>（公務・公用休暇）</t>
         </is>
       </c>
     </row>
     <row r="91" ht="32" customHeight="1">
       <c r="A91" s="27" t="inlineStr">
         <is>
-          <t>第16条　従業員が感染症に罹患し、医師の診断や法令に基づき出勤停止とされた場合は、その期間を休暇とする。賃金その他の取扱いは就業規則および賃金規程による。</t>
+          <t>第15条　従業員が裁判員、証人、選挙、官公庁の要請による職務に従事する場合は、その期間を休暇とする。</t>
         </is>
       </c>
     </row>
@@ -11092,317 +11341,394 @@
     <row r="93" ht="20" customHeight="1">
       <c r="A93" s="26" t="inlineStr">
         <is>
-          <t>（誕生日休暇）</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="20" customHeight="1">
+          <t>（感染症予防に伴う休暇）</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="32" customHeight="1">
       <c r="A94" s="27" t="inlineStr">
         <is>
-          <t>第17条　会社は、従業員に対し、誕生日月に1日の誕生日休暇を付与する。</t>
+          <t>第16条　従業員が感染症に罹患し、医師の診断や法令に基づき出勤停止とされた場合は、その期間を休暇とする。賃金その他の取扱いは就業規則および賃金規程による。</t>
         </is>
       </c>
     </row>
     <row r="95" ht="32" customHeight="1">
       <c r="A95" s="27" t="inlineStr">
         <is>
-          <t>2　シフト勤務等の都合により、従業員の希望がある場合は、誕生日に代えて前後の勤務日に振り替えることができる。</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="20" customHeight="1">
-      <c r="A96" s="27" t="inlineStr">
-        <is>
-          <t>3　誕生日休暇に伴う手当については「福利厚生規程」に定める。</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="8" customHeight="1"/>
-    <row r="98" ht="20" customHeight="1">
-      <c r="A98" s="26" t="inlineStr">
-        <is>
-          <t>（その他の特別休暇）</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="32" customHeight="1">
-      <c r="A99" s="27" t="inlineStr">
-        <is>
-          <t>第18条　会社は、災害その他社会的要請や会社が必要と認める場合に、特別休暇を付与することがある。</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="8" customHeight="1"/>
-    <row r="101" ht="8" customHeight="1">
-      <c r="A101" s="28" t="inlineStr"/>
-      <c r="B101" s="12" t="n"/>
-      <c r="C101" s="12" t="n"/>
-      <c r="D101" s="12" t="n"/>
-      <c r="E101" s="12" t="n"/>
-    </row>
-    <row r="102" ht="10" customHeight="1"/>
-    <row r="103" ht="30" customHeight="1">
-      <c r="A103" s="25" t="inlineStr">
-        <is>
-          <t>第4章　手続</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="20" customHeight="1">
-      <c r="A104" s="26" t="inlineStr">
-        <is>
-          <t>（申請手続）</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="32" customHeight="1">
-      <c r="A105" s="27" t="inlineStr">
-        <is>
-          <t>第19条　従業員は、休暇を取得しようとするときは、所定の様式により事前に申請し、上長の承認を得なければならない。ただし、やむを得ない場合は事後速やかに届け出る。</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="8" customHeight="1"/>
+          <t>2　法令に基づかず、会社の判断により出勤を停止させた場合は、労働基準法第26条に基づき休業手当（平均賃金の100分の60以上）を支払う。</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="8" customHeight="1"/>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="26" t="inlineStr">
+        <is>
+          <t>（生理休暇）</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="32" customHeight="1">
+      <c r="A98" s="27" t="inlineStr">
+        <is>
+          <t>第16条の2　生理日の就業が著しく困難な女性従業員が請求したときは、必要な期間の休暇を与える。</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="8" customHeight="1"/>
+    <row r="100" ht="20" customHeight="1">
+      <c r="A100" s="26" t="inlineStr">
+        <is>
+          <t>（育児時間）</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="32" customHeight="1">
+      <c r="A101" s="27" t="inlineStr">
+        <is>
+          <t>第16条の3　生後1年に達しない子を育てる女性従業員が請求したときは、休憩時間のほか1日2回、各30分の育児時間を与える。</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="8" customHeight="1"/>
+    <row r="103" ht="20" customHeight="1">
+      <c r="A103" s="26" t="inlineStr">
+        <is>
+          <t>（母性健康管理）</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="32" customHeight="1">
+      <c r="A104" s="27" t="inlineStr">
+        <is>
+          <t>第16条の4　妊娠中及び出産後1年以内の女性従業員が請求したときは、男女雇用機会均等法に基づき、保健指導または健康診査を受けるための時間を与える。</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="8" customHeight="1"/>
+    <row r="106" ht="20" customHeight="1">
+      <c r="A106" s="26" t="inlineStr">
+        <is>
+          <t>（誕生日休暇）</t>
+        </is>
+      </c>
+    </row>
     <row r="107" ht="20" customHeight="1">
-      <c r="A107" s="26" t="inlineStr">
-        <is>
-          <t>（診断書等の提出）</t>
+      <c r="A107" s="27" t="inlineStr">
+        <is>
+          <t>第17条　会社は、従業員に対し、誕生日月に1日の誕生日休暇を付与する。</t>
         </is>
       </c>
     </row>
     <row r="108" ht="32" customHeight="1">
       <c r="A108" s="27" t="inlineStr">
         <is>
-          <t>第20条　従業員は、次の場合に医師の診断書その他会社が認める証明書を提出しなければならない。</t>
+          <t>2　シフト勤務等の都合により、従業員の希望がある場合は、誕生日に代えて前後の勤務日に振り替えることができる。</t>
         </is>
       </c>
     </row>
     <row r="109" ht="20" customHeight="1">
       <c r="A109" s="27" t="inlineStr">
         <is>
+          <t>3　誕生日休暇に伴う手当については「福利厚生規程」に定める。</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="8" customHeight="1"/>
+    <row r="111" ht="20" customHeight="1">
+      <c r="A111" s="26" t="inlineStr">
+        <is>
+          <t>（その他の特別休暇）</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="32" customHeight="1">
+      <c r="A112" s="27" t="inlineStr">
+        <is>
+          <t>第18条　会社は、災害その他社会的要請や会社が必要と認める場合に、特別休暇を付与することがある。</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="8" customHeight="1"/>
+    <row r="114" ht="8" customHeight="1">
+      <c r="A114" s="28" t="inlineStr"/>
+      <c r="B114" s="12" t="n"/>
+      <c r="C114" s="12" t="n"/>
+      <c r="D114" s="12" t="n"/>
+      <c r="E114" s="12" t="n"/>
+    </row>
+    <row r="115" ht="10" customHeight="1"/>
+    <row r="116" ht="30" customHeight="1">
+      <c r="A116" s="25" t="inlineStr">
+        <is>
+          <t>第4章　手続</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="20" customHeight="1">
+      <c r="A117" s="26" t="inlineStr">
+        <is>
+          <t>（申請手続）</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="32" customHeight="1">
+      <c r="A118" s="27" t="inlineStr">
+        <is>
+          <t>第19条　従業員は、休暇を取得しようとするときは、所定の様式により事前に申請し、上長の承認を得なければならない。ただし、やむを得ない場合は事後速やかに届け出る。</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="8" customHeight="1"/>
+    <row r="120" ht="20" customHeight="1">
+      <c r="A120" s="26" t="inlineStr">
+        <is>
+          <t>（診断書等の提出）</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="32" customHeight="1">
+      <c r="A121" s="27" t="inlineStr">
+        <is>
+          <t>第20条　従業員は、次の場合に医師の診断書その他会社が認める証明書を提出しなければならない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="20" customHeight="1">
+      <c r="A122" s="27" t="inlineStr">
+        <is>
           <t>1　私傷病により連続して3日以上欠勤するとき</t>
         </is>
       </c>
     </row>
-    <row r="110" ht="20" customHeight="1">
-      <c r="A110" s="27" t="inlineStr">
+    <row r="123" ht="20" customHeight="1">
+      <c r="A123" s="27" t="inlineStr">
         <is>
           <t>2　休職を申請するとき</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="20" customHeight="1">
-      <c r="A111" s="27" t="inlineStr">
+    <row r="124" ht="20" customHeight="1">
+      <c r="A124" s="27" t="inlineStr">
         <is>
           <t>3　復職を希望するとき（精神疾患・適応障害・うつ病等を含む）</t>
         </is>
       </c>
     </row>
-    <row r="112" ht="20" customHeight="1">
-      <c r="A112" s="27" t="inlineStr">
+    <row r="125" ht="20" customHeight="1">
+      <c r="A125" s="27" t="inlineStr">
         <is>
           <t>4　産前産後休業、育児休業、介護休業、感染症罹患など、法令に基づく休暇を取得するとき</t>
         </is>
       </c>
     </row>
-    <row r="113" ht="20" customHeight="1">
-      <c r="A113" s="27" t="inlineStr">
+    <row r="126" ht="20" customHeight="1">
+      <c r="A126" s="27" t="inlineStr">
         <is>
           <t>5　会社が安全衛生管理上必要と認めたとき</t>
         </is>
       </c>
     </row>
-    <row r="114" ht="20" customHeight="1">
-      <c r="A114" s="27" t="inlineStr">
+    <row r="127" ht="20" customHeight="1">
+      <c r="A127" s="27" t="inlineStr">
         <is>
           <t>2　診断書等の作成費用は、原則として従業員の負担とする。</t>
         </is>
       </c>
     </row>
-    <row r="115" ht="20" customHeight="1">
-      <c r="A115" s="27" t="inlineStr">
+    <row r="128" ht="20" customHeight="1">
+      <c r="A128" s="27" t="inlineStr">
         <is>
           <t>3　ただし、次の各号に該当する場合は会社が費用を負担する。</t>
         </is>
       </c>
     </row>
-    <row r="116" ht="20" customHeight="1">
-      <c r="A116" s="27" t="inlineStr">
+    <row r="129" ht="20" customHeight="1">
+      <c r="A129" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">　1　会社が独自に必要と判断し、従業員の申請とは別に診断書その他の証明書を求めた場合</t>
         </is>
       </c>
     </row>
-    <row r="117" ht="20" customHeight="1">
-      <c r="A117" s="27" t="inlineStr">
+    <row r="130" ht="20" customHeight="1">
+      <c r="A130" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">　2　労働安全衛生法に基づく健康診断や再検査、特殊健康診断に関する場合</t>
         </is>
       </c>
     </row>
-    <row r="118" ht="20" customHeight="1">
-      <c r="A118" s="27" t="inlineStr">
+    <row r="131" ht="20" customHeight="1">
+      <c r="A131" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">　3　労災（業務災害・通勤災害）に関する診断書の場合</t>
         </is>
       </c>
     </row>
-    <row r="119" ht="8" customHeight="1"/>
-    <row r="120" ht="8" customHeight="1">
-      <c r="A120" s="28" t="inlineStr"/>
-      <c r="B120" s="12" t="n"/>
-      <c r="C120" s="12" t="n"/>
-      <c r="D120" s="12" t="n"/>
-      <c r="E120" s="12" t="n"/>
-    </row>
-    <row r="121" ht="10" customHeight="1"/>
-    <row r="122" ht="30" customHeight="1">
-      <c r="A122" s="25" t="inlineStr">
+    <row r="132" ht="8" customHeight="1"/>
+    <row r="133" ht="8" customHeight="1">
+      <c r="A133" s="28" t="inlineStr"/>
+      <c r="B133" s="12" t="n"/>
+      <c r="C133" s="12" t="n"/>
+      <c r="D133" s="12" t="n"/>
+      <c r="E133" s="12" t="n"/>
+    </row>
+    <row r="134" ht="10" customHeight="1"/>
+    <row r="135" ht="30" customHeight="1">
+      <c r="A135" s="25" t="inlineStr">
         <is>
           <t>第5章　その他</t>
         </is>
       </c>
     </row>
-    <row r="123" ht="20" customHeight="1">
-      <c r="A123" s="26" t="inlineStr">
+    <row r="136" ht="20" customHeight="1">
+      <c r="A136" s="26" t="inlineStr">
         <is>
           <t>（不利益取扱い禁止）</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="32" customHeight="1">
-      <c r="A124" s="27" t="inlineStr">
+    <row r="137" ht="32" customHeight="1">
+      <c r="A137" s="27" t="inlineStr">
         <is>
           <t>第21条　会社は、従業員が法令に基づく休暇または本規程による休暇を取得したことを理由として、不利益取扱いをしてはならない。</t>
         </is>
       </c>
     </row>
-    <row r="125" ht="8" customHeight="1"/>
-    <row r="126" ht="20" customHeight="1">
-      <c r="A126" s="26" t="inlineStr">
+    <row r="138" ht="8" customHeight="1"/>
+    <row r="139" ht="20" customHeight="1">
+      <c r="A139" s="26" t="inlineStr">
         <is>
           <t>（休暇中の待遇）</t>
         </is>
       </c>
     </row>
-    <row r="127" ht="32" customHeight="1">
-      <c r="A127" s="27" t="inlineStr">
+    <row r="140" ht="32" customHeight="1">
+      <c r="A140" s="27" t="inlineStr">
         <is>
           <t>第22条　休暇中の賃金、社会保険その他の待遇については、就業規則、賃金規程及び関係規程による。</t>
         </is>
       </c>
     </row>
-    <row r="128" ht="8" customHeight="1"/>
-    <row r="129" ht="8" customHeight="1">
-      <c r="A129" s="28" t="inlineStr"/>
-      <c r="B129" s="12" t="n"/>
-      <c r="C129" s="12" t="n"/>
-      <c r="D129" s="12" t="n"/>
-      <c r="E129" s="12" t="n"/>
-    </row>
-    <row r="130" ht="10" customHeight="1"/>
-    <row r="131" ht="30" customHeight="1">
-      <c r="A131" s="25" t="inlineStr">
+    <row r="141" ht="8" customHeight="1"/>
+    <row r="142" ht="8" customHeight="1">
+      <c r="A142" s="28" t="inlineStr"/>
+      <c r="B142" s="12" t="n"/>
+      <c r="C142" s="12" t="n"/>
+      <c r="D142" s="12" t="n"/>
+      <c r="E142" s="12" t="n"/>
+    </row>
+    <row r="143" ht="10" customHeight="1"/>
+    <row r="144" ht="30" customHeight="1">
+      <c r="A144" s="25" t="inlineStr">
         <is>
           <t>附則</t>
         </is>
       </c>
     </row>
-    <row r="132" ht="20" customHeight="1">
-      <c r="A132" s="27" t="inlineStr">
+    <row r="145" ht="20" customHeight="1">
+      <c r="A145" s="27" t="inlineStr">
         <is>
           <t>1　本規程に定めのない事項は、就業規則その他関係規程による。</t>
         </is>
       </c>
     </row>
-    <row r="133" ht="20" customHeight="1">
-      <c r="A133" s="27" t="inlineStr">
+    <row r="146" ht="20" customHeight="1">
+      <c r="A146" s="27" t="inlineStr">
         <is>
           <t>2　本規程は令和8年2月1日から施行する。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="84">
+  <mergeCells count="94">
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="A142:E142"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A45:E45"/>
     <mergeCell ref="A94:E94"/>
     <mergeCell ref="A103:E103"/>
+    <mergeCell ref="A79:E79"/>
     <mergeCell ref="A87:E87"/>
     <mergeCell ref="A65:E65"/>
+    <mergeCell ref="A128:E128"/>
+    <mergeCell ref="A137:E137"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="A46:E46"/>
-    <mergeCell ref="A105:E105"/>
+    <mergeCell ref="A136:E136"/>
     <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A57:E57"/>
-    <mergeCell ref="A113:E113"/>
+    <mergeCell ref="A139:E139"/>
     <mergeCell ref="A71:E71"/>
     <mergeCell ref="A129:E129"/>
     <mergeCell ref="A91:E91"/>
     <mergeCell ref="A131:E131"/>
+    <mergeCell ref="A100:E100"/>
     <mergeCell ref="A43:E43"/>
     <mergeCell ref="A52:E52"/>
     <mergeCell ref="A63:E63"/>
-    <mergeCell ref="A115:E115"/>
     <mergeCell ref="A93:E93"/>
+    <mergeCell ref="A130:E130"/>
     <mergeCell ref="A77:E77"/>
+    <mergeCell ref="A83:E83"/>
     <mergeCell ref="A49:E49"/>
-    <mergeCell ref="A132:E132"/>
     <mergeCell ref="A36:E36"/>
     <mergeCell ref="A69:E69"/>
-    <mergeCell ref="A78:E78"/>
     <mergeCell ref="A118:E118"/>
-    <mergeCell ref="A75:E75"/>
     <mergeCell ref="A133:E133"/>
     <mergeCell ref="A80:E80"/>
     <mergeCell ref="A120:E120"/>
+    <mergeCell ref="A55:E55"/>
     <mergeCell ref="A95:E95"/>
     <mergeCell ref="A104:E104"/>
-    <mergeCell ref="A81:E81"/>
+    <mergeCell ref="A97:E97"/>
+    <mergeCell ref="A106:E106"/>
     <mergeCell ref="A38:E38"/>
-    <mergeCell ref="A96:E96"/>
     <mergeCell ref="A31:E31"/>
     <mergeCell ref="A58:E58"/>
     <mergeCell ref="A40:E40"/>
     <mergeCell ref="A67:E67"/>
+    <mergeCell ref="A73:E73"/>
     <mergeCell ref="A82:E82"/>
+    <mergeCell ref="A60:E60"/>
     <mergeCell ref="A123:E123"/>
-    <mergeCell ref="A110:E110"/>
+    <mergeCell ref="A146:E146"/>
     <mergeCell ref="A124:E124"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A108:E108"/>
     <mergeCell ref="A84:E84"/>
     <mergeCell ref="A66:E66"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A135:E135"/>
+    <mergeCell ref="A144:E144"/>
     <mergeCell ref="A122:E122"/>
+    <mergeCell ref="A125:E125"/>
     <mergeCell ref="A72:E72"/>
     <mergeCell ref="A28:E28"/>
     <mergeCell ref="A112:E112"/>
+    <mergeCell ref="A121:E121"/>
     <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A44:E44"/>
     <mergeCell ref="A127:E127"/>
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A114:E114"/>
     <mergeCell ref="A59:E59"/>
-    <mergeCell ref="A64:E64"/>
     <mergeCell ref="A98:E98"/>
+    <mergeCell ref="A51:E51"/>
     <mergeCell ref="A107:E107"/>
     <mergeCell ref="A61:E61"/>
     <mergeCell ref="A88:E88"/>
     <mergeCell ref="A70:E70"/>
     <mergeCell ref="A54:E54"/>
-    <mergeCell ref="A41:E41"/>
     <mergeCell ref="A90:E90"/>
-    <mergeCell ref="A99:E99"/>
     <mergeCell ref="A74:E74"/>
     <mergeCell ref="A56:E56"/>
     <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A145:E145"/>
     <mergeCell ref="A101:E101"/>
+    <mergeCell ref="A76:E76"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="A85:E85"/>
     <mergeCell ref="A116:E116"/>
     <mergeCell ref="A126:E126"/>
-    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A140:E140"/>
     <mergeCell ref="A109:E109"/>
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A68:E68"/>

</xml_diff>

<commit_message>
感染症対策指針: set committee/training/drill months to June and November
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019FEKn7HFzGRhKMsA45fWaY
</commit_message>
<xml_diff>
--- a/output/いいかいご_契約書類一式.xlsx
+++ b/output/いいかいご_契約書類一式.xlsx
@@ -9186,7 +9186,7 @@
     <row r="64" ht="48" customHeight="1">
       <c r="A64" s="27" t="inlineStr">
         <is>
-          <t>感染対策委員会は、おおむね6か月に1回以上（4月・10月を予定）定期的に開催する。また、感染症発生時には、必要に応じて随時開催する。開催はテレビ電話装置等を活用して行うことができる。</t>
+          <t>感染対策委員会は、おおむね6か月に1回以上（6月・11月を予定）定期的に開催する。また、感染症発生時には、必要に応じて随時開催する。開催はテレビ電話装置等を活用して行うことができる。</t>
         </is>
       </c>
     </row>
@@ -9355,7 +9355,7 @@
       </c>
       <c r="B82" s="40" t="inlineStr">
         <is>
-          <t>5月・11月</t>
+          <t>6月・11月</t>
         </is>
       </c>
       <c r="C82" s="4" t="n"/>
@@ -9451,7 +9451,7 @@
       </c>
       <c r="B92" s="40" t="inlineStr">
         <is>
-          <t>5月</t>
+          <t>6月</t>
         </is>
       </c>
       <c r="C92" s="4" t="n"/>

</xml_diff>